<commit_message>
fix: Atualização diária dos dados
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CE16016-5FBA-486C-A349-0925041B09E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9AB6FD6-E1B2-41FE-BF51-4FB2D05427D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
   <sheets>
     <sheet name="FaturamentoBruto" sheetId="1" r:id="rId1"/>
@@ -1479,18 +1479,6 @@
     <xf numFmtId="4" fontId="20" fillId="33" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="34" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="34" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="4" fontId="19" fillId="33" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
@@ -1523,6 +1511,18 @@
     </xf>
     <xf numFmtId="4" fontId="19" fillId="33" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1900,7 +1900,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19101EBF-008C-4E37-90C0-CF2D419D5300}">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1909,16 +1909,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="48" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="50" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="40"/>
+      <c r="C1" s="51"/>
     </row>
     <row r="2" spans="1:3" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="38"/>
+      <c r="A2" s="49"/>
       <c r="B2" s="1" t="s">
         <v>78</v>
       </c>
@@ -2103,14 +2103,25 @@
       </c>
     </row>
     <row r="19" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="8">
+        <v>46316</v>
+      </c>
+      <c r="B19">
+        <v>548968.22</v>
+      </c>
+      <c r="C19">
+        <v>-24640.94</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B19" s="5">
-        <v>6314600.4000000004</v>
-      </c>
-      <c r="C19" s="5">
-        <v>-239616.11</v>
+      <c r="B20" s="5">
+        <v>6838785.3700000001</v>
+      </c>
+      <c r="C20" s="5">
+        <v>-264257.05</v>
       </c>
     </row>
   </sheetData>
@@ -2151,8 +2162,11 @@
     <hyperlink ref="B3" r:id="rId30" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=01%2F10%2F2026&amp;wDT_FIM=01%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{57C038F4-9037-4D9B-8567-B2DBF298F437}"/>
     <hyperlink ref="B18" r:id="rId31" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=20%2F10%2F2026&amp;wDT_FIM=20%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{03D2D6FF-12B4-4538-8F9C-83559C00711E}"/>
     <hyperlink ref="C18" r:id="rId32" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=20%2F10%2F2026&amp;wDT_FIM=20%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F40DF996-3027-4D6F-B560-A994ECD0B5DB}"/>
+    <hyperlink ref="B19" r:id="rId33" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=21%2F10%2F2026&amp;wDT_FIM=21%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{6866647E-AEF9-4707-8437-EEFD20D22BE1}"/>
+    <hyperlink ref="C19" r:id="rId34" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=21%2F10%2F2026&amp;wDT_FIM=21%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{86BC9795-12E6-4058-945B-DB513080C406}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId35"/>
 </worksheet>
 </file>
 
@@ -10826,13 +10840,13 @@
       <c r="A619" s="13">
         <v>46315</v>
       </c>
-      <c r="B619" s="45">
-        <v>101</v>
-      </c>
-      <c r="C619" s="46" t="s">
+      <c r="B619" s="41">
+        <v>101</v>
+      </c>
+      <c r="C619" s="42" t="s">
         <v>199</v>
       </c>
-      <c r="D619" s="47">
+      <c r="D619" s="43">
         <v>13323.95</v>
       </c>
     </row>
@@ -10840,13 +10854,13 @@
       <c r="A620" s="13">
         <v>46315</v>
       </c>
-      <c r="B620" s="48">
-        <v>101</v>
-      </c>
-      <c r="C620" s="42" t="s">
+      <c r="B620" s="44">
+        <v>101</v>
+      </c>
+      <c r="C620" s="38" t="s">
         <v>200</v>
       </c>
-      <c r="D620" s="43">
+      <c r="D620" s="39">
         <v>-55768.84</v>
       </c>
     </row>
@@ -10860,7 +10874,7 @@
       <c r="C621" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="D621" s="41">
+      <c r="D621" s="37">
         <v>55838.54</v>
       </c>
     </row>
@@ -10874,7 +10888,7 @@
       <c r="C622" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D622" s="41">
+      <c r="D622" s="37">
         <v>4080</v>
       </c>
     </row>
@@ -10888,7 +10902,7 @@
       <c r="C623" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D623" s="41">
+      <c r="D623" s="37">
         <v>3760.5</v>
       </c>
     </row>
@@ -10896,13 +10910,13 @@
       <c r="A624" s="13">
         <v>46315</v>
       </c>
-      <c r="B624" s="48">
-        <v>101</v>
-      </c>
-      <c r="C624" s="42" t="s">
+      <c r="B624" s="44">
+        <v>101</v>
+      </c>
+      <c r="C624" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="D624" s="43">
+      <c r="D624" s="39">
         <v>-3608</v>
       </c>
     </row>
@@ -10916,7 +10930,7 @@
       <c r="C625" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D625" s="41">
+      <c r="D625" s="37">
         <v>7985.15</v>
       </c>
     </row>
@@ -10930,7 +10944,7 @@
       <c r="C626" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D626" s="41">
+      <c r="D626" s="37">
         <v>2076.4699999999998</v>
       </c>
     </row>
@@ -10944,7 +10958,7 @@
       <c r="C627" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D627" s="41">
+      <c r="D627" s="37">
         <v>5557.21</v>
       </c>
     </row>
@@ -10958,7 +10972,7 @@
       <c r="C628" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D628" s="41">
+      <c r="D628" s="37">
         <v>13847.99</v>
       </c>
     </row>
@@ -10972,7 +10986,7 @@
       <c r="C629" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D629" s="44">
+      <c r="D629" s="40">
         <v>214.82</v>
       </c>
     </row>
@@ -10986,7 +11000,7 @@
       <c r="C630" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D630" s="41">
+      <c r="D630" s="37">
         <v>1716</v>
       </c>
     </row>
@@ -11000,7 +11014,7 @@
       <c r="C631" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D631" s="44">
+      <c r="D631" s="40">
         <v>544.82000000000005</v>
       </c>
     </row>
@@ -11014,7 +11028,7 @@
       <c r="C632" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D632" s="41">
+      <c r="D632" s="37">
         <v>1990</v>
       </c>
     </row>
@@ -11028,7 +11042,7 @@
       <c r="C633" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D633" s="41">
+      <c r="D633" s="37">
         <v>25886.46</v>
       </c>
     </row>
@@ -11042,7 +11056,7 @@
       <c r="C634" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="D634" s="44">
+      <c r="D634" s="40">
         <v>500.9</v>
       </c>
     </row>
@@ -11056,7 +11070,7 @@
       <c r="C635" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D635" s="44">
+      <c r="D635" s="40">
         <v>364.32</v>
       </c>
     </row>
@@ -11070,7 +11084,7 @@
       <c r="C636" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D636" s="41">
+      <c r="D636" s="37">
         <v>23277.06</v>
       </c>
     </row>
@@ -11084,7 +11098,7 @@
       <c r="C637" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D637" s="44">
+      <c r="D637" s="40">
         <v>513</v>
       </c>
     </row>
@@ -11098,7 +11112,7 @@
       <c r="C638" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D638" s="41">
+      <c r="D638" s="37">
         <v>21486.36</v>
       </c>
     </row>
@@ -11106,13 +11120,13 @@
       <c r="A639" s="13">
         <v>46315</v>
       </c>
-      <c r="B639" s="48">
-        <v>101</v>
-      </c>
-      <c r="C639" s="42" t="s">
+      <c r="B639" s="44">
+        <v>101</v>
+      </c>
+      <c r="C639" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="D639" s="43">
+      <c r="D639" s="39">
         <v>-3775.5</v>
       </c>
     </row>
@@ -11126,7 +11140,7 @@
       <c r="C640" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D640" s="41">
+      <c r="D640" s="37">
         <v>14512.3</v>
       </c>
     </row>
@@ -11140,7 +11154,7 @@
       <c r="C641" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D641" s="41">
+      <c r="D641" s="37">
         <v>10216.86</v>
       </c>
     </row>
@@ -11154,7 +11168,7 @@
       <c r="C642" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="D642" s="41">
+      <c r="D642" s="37">
         <v>3528.2</v>
       </c>
     </row>
@@ -11168,7 +11182,7 @@
       <c r="C643" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D643" s="41">
+      <c r="D643" s="37">
         <v>86365.37</v>
       </c>
     </row>
@@ -11182,7 +11196,7 @@
       <c r="C644" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D644" s="41">
+      <c r="D644" s="37">
         <v>7531.75</v>
       </c>
     </row>
@@ -11196,7 +11210,7 @@
       <c r="C645" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="D645" s="44">
+      <c r="D645" s="40">
         <v>642.16</v>
       </c>
     </row>
@@ -11210,7 +11224,7 @@
       <c r="C646" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D646" s="44">
+      <c r="D646" s="40">
         <v>616.14</v>
       </c>
     </row>
@@ -11224,7 +11238,7 @@
       <c r="C647" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D647" s="41">
+      <c r="D647" s="37">
         <v>4333.8900000000003</v>
       </c>
     </row>
@@ -11238,7 +11252,7 @@
       <c r="C648" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D648" s="41">
+      <c r="D648" s="37">
         <v>2112</v>
       </c>
     </row>
@@ -11252,7 +11266,7 @@
       <c r="C649" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D649" s="44">
+      <c r="D649" s="40">
         <v>697.32</v>
       </c>
     </row>
@@ -11266,7 +11280,7 @@
       <c r="C650" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D650" s="41">
+      <c r="D650" s="37">
         <v>2693.24</v>
       </c>
     </row>
@@ -11280,7 +11294,7 @@
       <c r="C651" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D651" s="41">
+      <c r="D651" s="37">
         <v>28127.439999999999</v>
       </c>
     </row>
@@ -11294,7 +11308,7 @@
       <c r="C652" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D652" s="41">
+      <c r="D652" s="37">
         <v>5268.9</v>
       </c>
     </row>
@@ -11308,7 +11322,7 @@
       <c r="C653" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D653" s="41">
+      <c r="D653" s="37">
         <v>3558</v>
       </c>
     </row>
@@ -11322,7 +11336,7 @@
       <c r="C654" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D654" s="41">
+      <c r="D654" s="37">
         <v>2771.7</v>
       </c>
     </row>
@@ -11336,7 +11350,7 @@
       <c r="C655" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D655" s="41">
+      <c r="D655" s="37">
         <v>2805.96</v>
       </c>
     </row>
@@ -11350,7 +11364,7 @@
       <c r="C656" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D656" s="41">
+      <c r="D656" s="37">
         <v>1170.45</v>
       </c>
     </row>
@@ -11364,7 +11378,7 @@
       <c r="C657" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D657" s="41">
+      <c r="D657" s="37">
         <v>1281.8399999999999</v>
       </c>
     </row>
@@ -11378,7 +11392,7 @@
       <c r="C658" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D658" s="41">
+      <c r="D658" s="37">
         <v>2782.44</v>
       </c>
     </row>
@@ -11392,7 +11406,7 @@
       <c r="C659" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D659" s="41">
+      <c r="D659" s="37">
         <v>1303.49</v>
       </c>
     </row>
@@ -11406,7 +11420,7 @@
       <c r="C660" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D660" s="41">
+      <c r="D660" s="37">
         <v>7547.3</v>
       </c>
     </row>
@@ -11420,7 +11434,7 @@
       <c r="C661" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D661" s="41">
+      <c r="D661" s="37">
         <v>14854.77</v>
       </c>
     </row>
@@ -11434,7 +11448,7 @@
       <c r="C662" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="D662" s="41">
+      <c r="D662" s="37">
         <v>6467.2</v>
       </c>
     </row>
@@ -11448,7 +11462,7 @@
       <c r="C663" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D663" s="44">
+      <c r="D663" s="40">
         <v>741</v>
       </c>
     </row>
@@ -11462,7 +11476,7 @@
       <c r="C664" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="D664" s="41">
+      <c r="D664" s="37">
         <v>1899.2</v>
       </c>
     </row>
@@ -11476,7 +11490,7 @@
       <c r="C665" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D665" s="44">
+      <c r="D665" s="40">
         <v>673.31</v>
       </c>
     </row>
@@ -11490,7 +11504,7 @@
       <c r="C666" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="D666" s="44">
+      <c r="D666" s="40">
         <v>43.04</v>
       </c>
     </row>
@@ -11504,7 +11518,7 @@
       <c r="C667" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D667" s="41">
+      <c r="D667" s="37">
         <v>1026.5899999999999</v>
       </c>
     </row>
@@ -11518,7 +11532,7 @@
       <c r="C668" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="D668" s="44">
+      <c r="D668" s="40">
         <v>511.5</v>
       </c>
     </row>
@@ -11532,7 +11546,7 @@
       <c r="C669" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D669" s="41">
+      <c r="D669" s="37">
         <v>1920</v>
       </c>
     </row>
@@ -11546,7 +11560,7 @@
       <c r="C670" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="D670" s="41">
+      <c r="D670" s="37">
         <v>1912.5</v>
       </c>
     </row>
@@ -11560,7 +11574,7 @@
       <c r="C671" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D671" s="41">
+      <c r="D671" s="37">
         <v>1021.5</v>
       </c>
     </row>
@@ -11574,7 +11588,7 @@
       <c r="C672" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="D672" s="41">
+      <c r="D672" s="37">
         <v>5005.8</v>
       </c>
     </row>
@@ -11588,7 +11602,7 @@
       <c r="C673" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D673" s="41">
+      <c r="D673" s="37">
         <v>68825.39</v>
       </c>
     </row>
@@ -11602,7 +11616,7 @@
       <c r="C674" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D674" s="44">
+      <c r="D674" s="40">
         <v>205.45</v>
       </c>
     </row>
@@ -11610,13 +11624,13 @@
       <c r="A675" s="13">
         <v>46315</v>
       </c>
-      <c r="B675" s="49">
-        <v>101</v>
-      </c>
-      <c r="C675" s="50" t="s">
+      <c r="B675" s="45">
+        <v>101</v>
+      </c>
+      <c r="C675" s="46" t="s">
         <v>70</v>
       </c>
-      <c r="D675" s="51">
+      <c r="D675" s="47">
         <v>14159.4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Atualização nos dados
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9AB6FD6-E1B2-41FE-BF51-4FB2D05427D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3914F6D3-88F0-4CEC-B685-CD3E109245BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
   <sheets>
     <sheet name="FaturamentoBruto" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="223">
   <si>
     <t>Filial</t>
   </si>
@@ -681,6 +681,15 @@
   </si>
   <si>
     <t>ARS ENSINO SUPERIOR</t>
+  </si>
+  <si>
+    <t>HOSP BARRA DOR I</t>
+  </si>
+  <si>
+    <t>H NOSSA SRA CONCEICA</t>
+  </si>
+  <si>
+    <t>COI CLINICA 39.086.1</t>
   </si>
 </sst>
 </file>
@@ -1371,7 +1380,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -1523,6 +1532,9 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -2172,16 +2184,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2872C95-5BBD-470F-BA44-E40722CF8AA3}">
-  <dimension ref="A1:D675"/>
+  <dimension ref="A1:D721"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.28515625" style="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.5703125" style="12" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.140625" style="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="12"/>
-    <col min="6" max="6" width="9.85546875" style="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="12"/>
+    <col min="5" max="5" width="9.85546875" style="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="12"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -11634,6 +11645,650 @@
         <v>14159.4</v>
       </c>
     </row>
+    <row r="676" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A676" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B676" s="12">
+        <v>101</v>
+      </c>
+      <c r="C676" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="D676" s="52">
+        <v>52362.9</v>
+      </c>
+    </row>
+    <row r="677" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A677" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B677" s="12">
+        <v>101</v>
+      </c>
+      <c r="C677" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="D677" s="12">
+        <v>733.5</v>
+      </c>
+    </row>
+    <row r="678" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A678" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B678" s="12">
+        <v>101</v>
+      </c>
+      <c r="C678" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="D678" s="12">
+        <v>539.01</v>
+      </c>
+    </row>
+    <row r="679" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A679" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B679" s="12">
+        <v>101</v>
+      </c>
+      <c r="C679" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="D679" s="12">
+        <v>650.49</v>
+      </c>
+    </row>
+    <row r="680" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A680" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B680" s="12">
+        <v>101</v>
+      </c>
+      <c r="C680" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="D680" s="12">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="681" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A681" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B681" s="12">
+        <v>101</v>
+      </c>
+      <c r="C681" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="D681" s="12">
+        <v>979.59</v>
+      </c>
+    </row>
+    <row r="682" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A682" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B682" s="12">
+        <v>101</v>
+      </c>
+      <c r="C682" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="D682" s="52">
+        <v>7699.01</v>
+      </c>
+    </row>
+    <row r="683" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A683" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B683" s="12">
+        <v>101</v>
+      </c>
+      <c r="C683" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="D683" s="52">
+        <v>4080</v>
+      </c>
+    </row>
+    <row r="684" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A684" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B684" s="12">
+        <v>101</v>
+      </c>
+      <c r="C684" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="D684" s="52">
+        <v>3760.5</v>
+      </c>
+    </row>
+    <row r="685" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A685" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B685" s="12">
+        <v>101</v>
+      </c>
+      <c r="C685" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D685" s="52">
+        <v>65871.62</v>
+      </c>
+    </row>
+    <row r="686" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A686" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B686" s="12">
+        <v>101</v>
+      </c>
+      <c r="C686" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="D686" s="12">
+        <v>239.53</v>
+      </c>
+    </row>
+    <row r="687" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A687" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B687" s="12">
+        <v>101</v>
+      </c>
+      <c r="C687" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D687" s="52">
+        <v>2965</v>
+      </c>
+    </row>
+    <row r="688" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A688" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B688" s="12">
+        <v>101</v>
+      </c>
+      <c r="C688" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D688" s="52">
+        <v>2836.51</v>
+      </c>
+    </row>
+    <row r="689" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A689" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B689" s="12">
+        <v>101</v>
+      </c>
+      <c r="C689" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D689" s="52">
+        <v>29025.5</v>
+      </c>
+    </row>
+    <row r="690" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A690" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B690" s="12">
+        <v>101</v>
+      </c>
+      <c r="C690" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D690" s="52">
+        <v>4968</v>
+      </c>
+    </row>
+    <row r="691" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A691" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B691" s="12">
+        <v>101</v>
+      </c>
+      <c r="C691" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D691" s="52">
+        <v>-1625</v>
+      </c>
+    </row>
+    <row r="692" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A692" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B692" s="12">
+        <v>101</v>
+      </c>
+      <c r="C692" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D692" s="12">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="693" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A693" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B693" s="12">
+        <v>101</v>
+      </c>
+      <c r="C693" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D693" s="52">
+        <v>2520</v>
+      </c>
+    </row>
+    <row r="694" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A694" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B694" s="12">
+        <v>101</v>
+      </c>
+      <c r="C694" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="D694" s="12">
+        <v>-500.9</v>
+      </c>
+    </row>
+    <row r="695" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A695" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B695" s="12">
+        <v>101</v>
+      </c>
+      <c r="C695" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="D695" s="52">
+        <v>5772.09</v>
+      </c>
+    </row>
+    <row r="696" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A696" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B696" s="12">
+        <v>101</v>
+      </c>
+      <c r="C696" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D696" s="52">
+        <v>1091.42</v>
+      </c>
+    </row>
+    <row r="697" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A697" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B697" s="12">
+        <v>101</v>
+      </c>
+      <c r="C697" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D697" s="52">
+        <v>13836.2</v>
+      </c>
+    </row>
+    <row r="698" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A698" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B698" s="12">
+        <v>101</v>
+      </c>
+      <c r="C698" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="D698" s="52">
+        <v>3891.09</v>
+      </c>
+    </row>
+    <row r="699" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A699" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B699" s="12">
+        <v>101</v>
+      </c>
+      <c r="C699" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D699" s="52">
+        <v>-7027.68</v>
+      </c>
+    </row>
+    <row r="700" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A700" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B700" s="12">
+        <v>101</v>
+      </c>
+      <c r="C700" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D700" s="52">
+        <v>26872.07</v>
+      </c>
+    </row>
+    <row r="701" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A701" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B701" s="12">
+        <v>101</v>
+      </c>
+      <c r="C701" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="D701" s="52">
+        <v>11888.17</v>
+      </c>
+    </row>
+    <row r="702" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A702" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B702" s="12">
+        <v>101</v>
+      </c>
+      <c r="C702" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="D702" s="52">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="703" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A703" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B703" s="12">
+        <v>101</v>
+      </c>
+      <c r="C703" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="D703" s="52">
+        <v>-10339.959999999999</v>
+      </c>
+    </row>
+    <row r="704" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A704" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B704" s="12">
+        <v>101</v>
+      </c>
+      <c r="C704" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D704" s="52">
+        <v>1533.96</v>
+      </c>
+    </row>
+    <row r="705" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A705" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B705" s="12">
+        <v>101</v>
+      </c>
+      <c r="C705" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D705" s="52">
+        <v>3617.46</v>
+      </c>
+    </row>
+    <row r="706" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A706" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B706" s="12">
+        <v>101</v>
+      </c>
+      <c r="C706" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="D706" s="52">
+        <v>-5147.3999999999996</v>
+      </c>
+    </row>
+    <row r="707" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A707" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B707" s="12">
+        <v>101</v>
+      </c>
+      <c r="C707" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="D707" s="52">
+        <v>81796.06</v>
+      </c>
+    </row>
+    <row r="708" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A708" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B708" s="12">
+        <v>101</v>
+      </c>
+      <c r="C708" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D708" s="52">
+        <v>1639.96</v>
+      </c>
+    </row>
+    <row r="709" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A709" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B709" s="12">
+        <v>101</v>
+      </c>
+      <c r="C709" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D709" s="12">
+        <v>697.32</v>
+      </c>
+    </row>
+    <row r="710" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A710" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B710" s="12">
+        <v>101</v>
+      </c>
+      <c r="C710" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D710" s="52">
+        <v>28127.439999999999</v>
+      </c>
+    </row>
+    <row r="711" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A711" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B711" s="12">
+        <v>101</v>
+      </c>
+      <c r="C711" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D711" s="52">
+        <v>11770.06</v>
+      </c>
+    </row>
+    <row r="712" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A712" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B712" s="12">
+        <v>101</v>
+      </c>
+      <c r="C712" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D712" s="52">
+        <v>4590.1400000000003</v>
+      </c>
+    </row>
+    <row r="713" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A713" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B713" s="12">
+        <v>101</v>
+      </c>
+      <c r="C713" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="D713" s="52">
+        <v>8070.92</v>
+      </c>
+    </row>
+    <row r="714" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A714" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B714" s="12">
+        <v>101</v>
+      </c>
+      <c r="C714" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="D714" s="52">
+        <v>17442.8</v>
+      </c>
+    </row>
+    <row r="715" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A715" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B715" s="12">
+        <v>101</v>
+      </c>
+      <c r="C715" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D715" s="12">
+        <v>598.83000000000004</v>
+      </c>
+    </row>
+    <row r="716" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A716" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B716" s="12">
+        <v>101</v>
+      </c>
+      <c r="C716" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D716" s="52">
+        <v>80536.3</v>
+      </c>
+    </row>
+    <row r="717" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A717" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B717" s="12">
+        <v>101</v>
+      </c>
+      <c r="C717" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D717" s="52">
+        <v>54056.1</v>
+      </c>
+    </row>
+    <row r="718" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A718" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B718" s="12">
+        <v>101</v>
+      </c>
+      <c r="C718" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D718" s="52">
+        <v>5345.41</v>
+      </c>
+    </row>
+    <row r="719" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A719" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B719" s="12">
+        <v>101</v>
+      </c>
+      <c r="C719" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D719" s="52">
+        <v>1728.45</v>
+      </c>
+    </row>
+    <row r="720" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A720" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B720" s="12">
+        <v>101</v>
+      </c>
+      <c r="C720" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D720" s="52">
+        <v>1588.1</v>
+      </c>
+    </row>
+    <row r="721" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A721" s="13">
+        <v>46316</v>
+      </c>
+      <c r="B721" s="12">
+        <v>101</v>
+      </c>
+      <c r="C721" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D721" s="12">
+        <v>417.71</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Atualizãção diária dos dados
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CC3B8B4-8BBC-4146-BB53-D833FA4AFBB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF1DBFB3-004B-4660-AC17-7BDBDD53D6EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
@@ -1071,7 +1071,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -1231,6 +1231,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDEE2E6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1276,7 +1291,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1299,6 +1314,9 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="19" fillId="33" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1675,7 +1693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19101EBF-008C-4E37-90C0-CF2D419D5300}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15.75" thickBottom="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="3" bestFit="1" customWidth="1"/>
@@ -1902,21 +1920,32 @@
         <v>46318</v>
       </c>
       <c r="B21">
-        <v>369121.69</v>
+        <v>380210.58</v>
       </c>
       <c r="C21">
-        <v>-728.82</v>
+        <v>-19833.009999999998</v>
       </c>
     </row>
     <row r="22" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="9">
+        <v>46321</v>
+      </c>
+      <c r="B22">
+        <v>187326.15</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B22" s="2">
-        <v>7855067.1399999997</v>
-      </c>
-      <c r="C22" s="2">
-        <v>-291673.07</v>
+      <c r="B23" s="2">
+        <v>8053482.1799999997</v>
+      </c>
+      <c r="C23" s="2">
+        <v>-310777.26</v>
       </c>
     </row>
   </sheetData>
@@ -1955,11 +1984,13 @@
     <hyperlink ref="C18" r:id="rId32" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=20%2F10%2F2026&amp;wDT_FIM=20%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F40DF996-3027-4D6F-B560-A994ECD0B5DB}"/>
     <hyperlink ref="B19" r:id="rId33" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=21%2F10%2F2026&amp;wDT_FIM=21%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{6866647E-AEF9-4707-8437-EEFD20D22BE1}"/>
     <hyperlink ref="C19" r:id="rId34" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=21%2F10%2F2026&amp;wDT_FIM=21%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{86BC9795-12E6-4058-945B-DB513080C406}"/>
-    <hyperlink ref="B21" r:id="rId35" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{8AC67425-6A9D-4CE6-BE58-59016843D5F9}"/>
-    <hyperlink ref="C21" r:id="rId36" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{D7178C55-B681-4C63-9551-790DB0963D8A}"/>
+    <hyperlink ref="B21" r:id="rId35" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{ABF3F658-C78C-46C1-A6A0-EACB1F1312FC}"/>
+    <hyperlink ref="C21" r:id="rId36" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{A5E30353-68AD-4555-A4A4-F43F7F15A167}"/>
+    <hyperlink ref="B22" r:id="rId37" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{6A546647-FE3F-4BCF-9E75-A6F5618DE61E}"/>
+    <hyperlink ref="C22" r:id="rId38" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{67F55B4C-CA3E-4682-89A5-7FB10930EF0B}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId37"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId39"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: Atualização dos dados faltantes
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF1DBFB3-004B-4660-AC17-7BDBDD53D6EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7066F92A-3C54-4E55-B093-4C70A5EBDB1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
   <sheets>
     <sheet name="FaturamentoBruto" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="793" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="236">
   <si>
     <t>Filial</t>
   </si>
@@ -723,6 +723,12 @@
   </si>
   <si>
     <t>ALTHAIA</t>
+  </si>
+  <si>
+    <t>SECONCI CENTRO</t>
+  </si>
+  <si>
+    <t>DASA UNIDADE CENTRAL</t>
   </si>
 </sst>
 </file>
@@ -1996,7 +2002,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2872C95-5BBD-470F-BA44-E40722CF8AA3}">
-  <dimension ref="A1:D785"/>
+  <dimension ref="A1:D837"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="5" bestFit="1" customWidth="1"/>
@@ -12997,6 +13003,734 @@
         <v>2043.13</v>
       </c>
     </row>
+    <row r="786" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A786" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B786" s="5">
+        <v>101</v>
+      </c>
+      <c r="C786" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="D786" s="8">
+        <v>6482.29</v>
+      </c>
+    </row>
+    <row r="787" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A787" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B787" s="5">
+        <v>101</v>
+      </c>
+      <c r="C787" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="D787" s="8">
+        <v>3734.99</v>
+      </c>
+    </row>
+    <row r="788" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A788" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B788" s="5">
+        <v>101</v>
+      </c>
+      <c r="C788" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D788" s="8">
+        <v>3388.45</v>
+      </c>
+    </row>
+    <row r="789" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A789" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B789" s="5">
+        <v>101</v>
+      </c>
+      <c r="C789" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D789" s="8">
+        <v>1830.25</v>
+      </c>
+    </row>
+    <row r="790" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A790" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B790" s="5">
+        <v>101</v>
+      </c>
+      <c r="C790" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="D790" s="8">
+        <v>4233.4399999999996</v>
+      </c>
+    </row>
+    <row r="791" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A791" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B791" s="5">
+        <v>101</v>
+      </c>
+      <c r="C791" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D791" s="8">
+        <v>2359.8200000000002</v>
+      </c>
+    </row>
+    <row r="792" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A792" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B792" s="5">
+        <v>101</v>
+      </c>
+      <c r="C792" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="D792" s="8">
+        <v>62.38</v>
+      </c>
+    </row>
+    <row r="793" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A793" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B793" s="5">
+        <v>101</v>
+      </c>
+      <c r="C793" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D793" s="8">
+        <v>18390.54</v>
+      </c>
+    </row>
+    <row r="794" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A794" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B794" s="5">
+        <v>101</v>
+      </c>
+      <c r="C794" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="D794" s="8">
+        <v>-5109.24</v>
+      </c>
+    </row>
+    <row r="795" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A795" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B795" s="5">
+        <v>101</v>
+      </c>
+      <c r="C795" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D795" s="8">
+        <v>1169.6300000000001</v>
+      </c>
+    </row>
+    <row r="796" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A796" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B796" s="5">
+        <v>101</v>
+      </c>
+      <c r="C796" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D796" s="8">
+        <v>4069.44</v>
+      </c>
+    </row>
+    <row r="797" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A797" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B797" s="5">
+        <v>101</v>
+      </c>
+      <c r="C797" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D797" s="8">
+        <v>6860.52</v>
+      </c>
+    </row>
+    <row r="798" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A798" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B798" s="5">
+        <v>101</v>
+      </c>
+      <c r="C798" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D798" s="8">
+        <v>17075.599999999999</v>
+      </c>
+    </row>
+    <row r="799" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A799" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B799" s="5">
+        <v>101</v>
+      </c>
+      <c r="C799" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D799" s="8">
+        <v>629.70000000000005</v>
+      </c>
+    </row>
+    <row r="800" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A800" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B800" s="5">
+        <v>101</v>
+      </c>
+      <c r="C800" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D800" s="8">
+        <v>23280</v>
+      </c>
+    </row>
+    <row r="801" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A801" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B801" s="5">
+        <v>101</v>
+      </c>
+      <c r="C801" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D801" s="8">
+        <v>-14507.95</v>
+      </c>
+    </row>
+    <row r="802" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A802" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B802" s="5">
+        <v>101</v>
+      </c>
+      <c r="C802" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D802" s="8">
+        <v>30772.58</v>
+      </c>
+    </row>
+    <row r="803" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A803" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B803" s="5">
+        <v>101</v>
+      </c>
+      <c r="C803" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D803" s="8">
+        <v>4565.7700000000004</v>
+      </c>
+    </row>
+    <row r="804" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A804" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B804" s="5">
+        <v>101</v>
+      </c>
+      <c r="C804" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D804" s="8">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="805" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A805" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B805" s="5">
+        <v>101</v>
+      </c>
+      <c r="C805" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D805" s="8">
+        <v>3718.6</v>
+      </c>
+    </row>
+    <row r="806" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A806" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B806" s="5">
+        <v>101</v>
+      </c>
+      <c r="C806" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D806" s="8">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="807" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A807" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B807" s="5">
+        <v>101</v>
+      </c>
+      <c r="C807" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D807" s="8">
+        <v>23535.3</v>
+      </c>
+    </row>
+    <row r="808" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A808" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B808" s="5">
+        <v>101</v>
+      </c>
+      <c r="C808" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="D808" s="8">
+        <v>1324.51</v>
+      </c>
+    </row>
+    <row r="809" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A809" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B809" s="5">
+        <v>101</v>
+      </c>
+      <c r="C809" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D809" s="8">
+        <v>2430.8000000000002</v>
+      </c>
+    </row>
+    <row r="810" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A810" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B810" s="5">
+        <v>101</v>
+      </c>
+      <c r="C810" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D810" s="8">
+        <v>9221</v>
+      </c>
+    </row>
+    <row r="811" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A811" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B811" s="5">
+        <v>101</v>
+      </c>
+      <c r="C811" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D811" s="8">
+        <v>1003.3</v>
+      </c>
+    </row>
+    <row r="812" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A812" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B812" s="5">
+        <v>101</v>
+      </c>
+      <c r="C812" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D812" s="8">
+        <v>1186.92</v>
+      </c>
+    </row>
+    <row r="813" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A813" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B813" s="5">
+        <v>101</v>
+      </c>
+      <c r="C813" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D813" s="8">
+        <v>4779.62</v>
+      </c>
+    </row>
+    <row r="814" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A814" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B814" s="5">
+        <v>101</v>
+      </c>
+      <c r="C814" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D814" s="8">
+        <v>7.55</v>
+      </c>
+    </row>
+    <row r="815" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A815" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B815" s="5">
+        <v>101</v>
+      </c>
+      <c r="C815" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D815" s="8">
+        <v>1836.69</v>
+      </c>
+    </row>
+    <row r="816" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A816" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B816" s="5">
+        <v>101</v>
+      </c>
+      <c r="C816" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D816" s="8">
+        <v>1251.8499999999999</v>
+      </c>
+    </row>
+    <row r="817" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A817" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B817" s="5">
+        <v>101</v>
+      </c>
+      <c r="C817" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D817" s="8">
+        <v>562.20000000000005</v>
+      </c>
+    </row>
+    <row r="818" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A818" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B818" s="5">
+        <v>101</v>
+      </c>
+      <c r="C818" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D818" s="8">
+        <v>2790.95</v>
+      </c>
+    </row>
+    <row r="819" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A819" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B819" s="5">
+        <v>101</v>
+      </c>
+      <c r="C819" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D819" s="8">
+        <v>18450.2</v>
+      </c>
+    </row>
+    <row r="820" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A820" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B820" s="5">
+        <v>101</v>
+      </c>
+      <c r="C820" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D820" s="8">
+        <v>1783.2</v>
+      </c>
+    </row>
+    <row r="821" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A821" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B821" s="5">
+        <v>101</v>
+      </c>
+      <c r="C821" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="D821" s="8">
+        <v>1808.11</v>
+      </c>
+    </row>
+    <row r="822" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A822" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B822" s="5">
+        <v>101</v>
+      </c>
+      <c r="C822" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D822" s="8">
+        <v>469.15</v>
+      </c>
+    </row>
+    <row r="823" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A823" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B823" s="5">
+        <v>101</v>
+      </c>
+      <c r="C823" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D823" s="8">
+        <v>2848.8</v>
+      </c>
+    </row>
+    <row r="824" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A824" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B824" s="5">
+        <v>101</v>
+      </c>
+      <c r="C824" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D824" s="8">
+        <v>760.2</v>
+      </c>
+    </row>
+    <row r="825" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A825" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B825" s="5">
+        <v>101</v>
+      </c>
+      <c r="C825" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D825" s="8">
+        <v>2538.0500000000002</v>
+      </c>
+    </row>
+    <row r="826" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A826" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B826" s="5">
+        <v>101</v>
+      </c>
+      <c r="C826" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D826" s="8">
+        <v>1276.1199999999999</v>
+      </c>
+    </row>
+    <row r="827" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A827" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B827" s="5">
+        <v>101</v>
+      </c>
+      <c r="C827" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="D827" s="8">
+        <v>1478.7</v>
+      </c>
+    </row>
+    <row r="828" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A828" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B828" s="5">
+        <v>101</v>
+      </c>
+      <c r="C828" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D828" s="8">
+        <v>1573.78</v>
+      </c>
+    </row>
+    <row r="829" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A829" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B829" s="5">
+        <v>101</v>
+      </c>
+      <c r="C829" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D829" s="8">
+        <v>1705.41</v>
+      </c>
+    </row>
+    <row r="830" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A830" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B830" s="5">
+        <v>101</v>
+      </c>
+      <c r="C830" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D830" s="8">
+        <v>14430</v>
+      </c>
+    </row>
+    <row r="831" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A831" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B831" s="5">
+        <v>101</v>
+      </c>
+      <c r="C831" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="D831" s="8">
+        <v>4320</v>
+      </c>
+    </row>
+    <row r="832" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A832" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B832" s="5">
+        <v>101</v>
+      </c>
+      <c r="C832" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D832" s="8">
+        <v>122850</v>
+      </c>
+    </row>
+    <row r="833" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A833" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B833" s="5">
+        <v>101</v>
+      </c>
+      <c r="C833" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D833" s="8">
+        <v>-215.82</v>
+      </c>
+    </row>
+    <row r="834" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A834" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B834" s="5">
+        <v>101</v>
+      </c>
+      <c r="C834" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D834" s="8">
+        <v>1666.25</v>
+      </c>
+    </row>
+    <row r="835" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A835" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B835" s="5">
+        <v>101</v>
+      </c>
+      <c r="C835" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D835" s="8">
+        <v>4412.2</v>
+      </c>
+    </row>
+    <row r="836" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A836" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B836" s="5">
+        <v>101</v>
+      </c>
+      <c r="C836" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D836" s="8">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="837" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A837" s="6">
+        <v>46318</v>
+      </c>
+      <c r="B837" s="5">
+        <v>101</v>
+      </c>
+      <c r="C837" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D837" s="8">
+        <v>14134.72</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Atualização nos dados diários
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7066F92A-3C54-4E55-B093-4C70A5EBDB1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE0B3E1-62E1-44BA-B87A-0B3E5F518935}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
   <sheets>
     <sheet name="FaturamentoBruto" sheetId="1" r:id="rId1"/>
@@ -1077,7 +1077,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1237,21 +1237,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF808080"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFDEE2E6"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF808080"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF808080"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1297,7 +1282,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1320,9 +1305,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="19" fillId="33" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1703,7 +1685,7 @@
   <sheetFormatPr defaultRowHeight="15.75" thickBottom="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1933,11 +1915,11 @@
       </c>
     </row>
     <row r="22" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="9">
+      <c r="A22" s="3">
         <v>46321</v>
       </c>
       <c r="B22">
-        <v>187326.15</v>
+        <v>690331.86</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -1948,7 +1930,7 @@
         <v>75</v>
       </c>
       <c r="B23" s="2">
-        <v>8053482.1799999997</v>
+        <v>8556487.8900000006</v>
       </c>
       <c r="C23" s="2">
         <v>-310777.26</v>
@@ -1992,8 +1974,8 @@
     <hyperlink ref="C19" r:id="rId34" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=21%2F10%2F2026&amp;wDT_FIM=21%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{86BC9795-12E6-4058-945B-DB513080C406}"/>
     <hyperlink ref="B21" r:id="rId35" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{ABF3F658-C78C-46C1-A6A0-EACB1F1312FC}"/>
     <hyperlink ref="C21" r:id="rId36" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{A5E30353-68AD-4555-A4A4-F43F7F15A167}"/>
-    <hyperlink ref="B22" r:id="rId37" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{6A546647-FE3F-4BCF-9E75-A6F5618DE61E}"/>
-    <hyperlink ref="C22" r:id="rId38" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{67F55B4C-CA3E-4682-89A5-7FB10930EF0B}"/>
+    <hyperlink ref="B22" r:id="rId37" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{C4F5F9A5-AC8F-4808-8572-70D87C9D82F9}"/>
+    <hyperlink ref="C22" r:id="rId38" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{FD324AB2-9D0D-4917-8ADD-F06162E9FBEA}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId39"/>

</xml_diff>

<commit_message>
Atualização diária dos dados
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE0B3E1-62E1-44BA-B87A-0B3E5F518935}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F094D1D-294F-414B-BFEC-A1DEC515B7D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
   <sheets>
     <sheet name="FaturamentoBruto" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="242">
   <si>
     <t>Filial</t>
   </si>
@@ -729,6 +729,24 @@
   </si>
   <si>
     <t>DASA UNIDADE CENTRAL</t>
+  </si>
+  <si>
+    <t>WCA DO BRASIL</t>
+  </si>
+  <si>
+    <t>TRE TRIBUNAL</t>
+  </si>
+  <si>
+    <t>LAB SANTA LUZIA</t>
+  </si>
+  <si>
+    <t>HOSP HELIOPOLIS</t>
+  </si>
+  <si>
+    <t>DASA LAB HORMON</t>
+  </si>
+  <si>
+    <t>DASA 61.486.650/0686</t>
   </si>
 </sst>
 </file>
@@ -1681,7 +1699,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19101EBF-008C-4E37-90C0-CF2D419D5300}">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15.75" thickBottom="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="3" bestFit="1" customWidth="1"/>
@@ -1919,21 +1937,32 @@
         <v>46321</v>
       </c>
       <c r="B22">
-        <v>690331.86</v>
+        <v>833062.77</v>
       </c>
       <c r="C22">
+        <v>-8601.89</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
+        <v>46322</v>
+      </c>
+      <c r="B23">
+        <v>146303.18</v>
+      </c>
+      <c r="C23">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
+    <row r="24" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B23" s="2">
-        <v>8556487.8900000006</v>
-      </c>
-      <c r="C23" s="2">
-        <v>-310777.26</v>
+      <c r="B24" s="2">
+        <v>8845521.9800000004</v>
+      </c>
+      <c r="C24" s="2">
+        <v>-319379.15000000002</v>
       </c>
     </row>
   </sheetData>
@@ -1974,17 +2003,19 @@
     <hyperlink ref="C19" r:id="rId34" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=21%2F10%2F2026&amp;wDT_FIM=21%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{86BC9795-12E6-4058-945B-DB513080C406}"/>
     <hyperlink ref="B21" r:id="rId35" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{ABF3F658-C78C-46C1-A6A0-EACB1F1312FC}"/>
     <hyperlink ref="C21" r:id="rId36" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{A5E30353-68AD-4555-A4A4-F43F7F15A167}"/>
-    <hyperlink ref="B22" r:id="rId37" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{C4F5F9A5-AC8F-4808-8572-70D87C9D82F9}"/>
-    <hyperlink ref="C22" r:id="rId38" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{FD324AB2-9D0D-4917-8ADD-F06162E9FBEA}"/>
+    <hyperlink ref="B22" r:id="rId37" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F5D8DE54-95D1-46C8-88FE-0455E31F55EA}"/>
+    <hyperlink ref="C22" r:id="rId38" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{B6508494-A2ED-45CE-A06F-52BAF7398889}"/>
+    <hyperlink ref="B23" r:id="rId39" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{E234A0FC-3F1D-4E49-89FE-CFF8150000F6}"/>
+    <hyperlink ref="C23" r:id="rId40" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{3AB773AA-3A9E-4C38-8792-28BC2A833A14}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId39"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId41"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2872C95-5BBD-470F-BA44-E40722CF8AA3}">
-  <dimension ref="A1:D837"/>
+  <dimension ref="A1:D890"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="5" bestFit="1" customWidth="1"/>
@@ -13713,6 +13744,748 @@
         <v>14134.72</v>
       </c>
     </row>
+    <row r="838" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A838" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B838" s="5">
+        <v>101</v>
+      </c>
+      <c r="C838" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="D838" s="8">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="839" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A839" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B839" s="5">
+        <v>101</v>
+      </c>
+      <c r="C839" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="D839" s="8">
+        <v>128598.54</v>
+      </c>
+    </row>
+    <row r="840" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A840" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B840" s="5">
+        <v>101</v>
+      </c>
+      <c r="C840" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="D840" s="8">
+        <v>8212.14</v>
+      </c>
+    </row>
+    <row r="841" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A841" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B841" s="5">
+        <v>101</v>
+      </c>
+      <c r="C841" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="D841" s="8">
+        <v>2480.7600000000002</v>
+      </c>
+    </row>
+    <row r="842" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A842" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B842" s="5">
+        <v>101</v>
+      </c>
+      <c r="C842" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="D842" s="8">
+        <v>690.3</v>
+      </c>
+    </row>
+    <row r="843" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A843" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B843" s="5">
+        <v>101</v>
+      </c>
+      <c r="C843" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="D843" s="8">
+        <v>4145.6400000000003</v>
+      </c>
+    </row>
+    <row r="844" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A844" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B844" s="5">
+        <v>101</v>
+      </c>
+      <c r="C844" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="D844" s="8">
+        <v>2647.33</v>
+      </c>
+    </row>
+    <row r="845" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A845" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B845" s="5">
+        <v>101</v>
+      </c>
+      <c r="C845" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D845" s="8">
+        <v>9171.9</v>
+      </c>
+    </row>
+    <row r="846" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A846" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B846" s="5">
+        <v>101</v>
+      </c>
+      <c r="C846" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D846" s="8">
+        <v>2574.64</v>
+      </c>
+    </row>
+    <row r="847" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A847" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B847" s="5">
+        <v>101</v>
+      </c>
+      <c r="C847" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D847" s="8">
+        <v>567.6</v>
+      </c>
+    </row>
+    <row r="848" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A848" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B848" s="5">
+        <v>101</v>
+      </c>
+      <c r="C848" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D848" s="8">
+        <v>1511.02</v>
+      </c>
+    </row>
+    <row r="849" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A849" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B849" s="5">
+        <v>101</v>
+      </c>
+      <c r="C849" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D849" s="8">
+        <v>23563.1</v>
+      </c>
+    </row>
+    <row r="850" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A850" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B850" s="5">
+        <v>101</v>
+      </c>
+      <c r="C850" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D850" s="8">
+        <v>-761.75</v>
+      </c>
+    </row>
+    <row r="851" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A851" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B851" s="5">
+        <v>101</v>
+      </c>
+      <c r="C851" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D851" s="8">
+        <v>1582.08</v>
+      </c>
+    </row>
+    <row r="852" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A852" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B852" s="5">
+        <v>101</v>
+      </c>
+      <c r="C852" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="D852" s="8">
+        <v>1273.5</v>
+      </c>
+    </row>
+    <row r="853" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A853" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B853" s="5">
+        <v>101</v>
+      </c>
+      <c r="C853" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D853" s="8">
+        <v>-639.84</v>
+      </c>
+    </row>
+    <row r="854" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A854" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B854" s="5">
+        <v>101</v>
+      </c>
+      <c r="C854" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D854" s="8">
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="855" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A855" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B855" s="5">
+        <v>101</v>
+      </c>
+      <c r="C855" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D855" s="8">
+        <v>14381.87</v>
+      </c>
+    </row>
+    <row r="856" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A856" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B856" s="5">
+        <v>101</v>
+      </c>
+      <c r="C856" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D856" s="8">
+        <v>-3373.44</v>
+      </c>
+    </row>
+    <row r="857" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A857" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B857" s="5">
+        <v>101</v>
+      </c>
+      <c r="C857" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D857" s="8">
+        <v>5353.44</v>
+      </c>
+    </row>
+    <row r="858" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A858" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B858" s="5">
+        <v>101</v>
+      </c>
+      <c r="C858" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D858" s="8">
+        <v>5562.9</v>
+      </c>
+    </row>
+    <row r="859" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A859" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B859" s="5">
+        <v>101</v>
+      </c>
+      <c r="C859" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D859" s="8">
+        <v>20711.900000000001</v>
+      </c>
+    </row>
+    <row r="860" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A860" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B860" s="5">
+        <v>101</v>
+      </c>
+      <c r="C860" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="D860" s="8">
+        <v>9800</v>
+      </c>
+    </row>
+    <row r="861" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A861" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B861" s="5">
+        <v>101</v>
+      </c>
+      <c r="C861" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D861" s="8">
+        <v>-2700</v>
+      </c>
+    </row>
+    <row r="862" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A862" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B862" s="5">
+        <v>101</v>
+      </c>
+      <c r="C862" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D862" s="8">
+        <v>216623.32</v>
+      </c>
+    </row>
+    <row r="863" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A863" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B863" s="5">
+        <v>101</v>
+      </c>
+      <c r="C863" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D863" s="8">
+        <v>5527.5</v>
+      </c>
+    </row>
+    <row r="864" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A864" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B864" s="5">
+        <v>101</v>
+      </c>
+      <c r="C864" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D864" s="8">
+        <v>2108.84</v>
+      </c>
+    </row>
+    <row r="865" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A865" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B865" s="5">
+        <v>101</v>
+      </c>
+      <c r="C865" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D865" s="8">
+        <v>24648.5</v>
+      </c>
+    </row>
+    <row r="866" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A866" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B866" s="5">
+        <v>101</v>
+      </c>
+      <c r="C866" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D866" s="8">
+        <v>4589.7</v>
+      </c>
+    </row>
+    <row r="867" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A867" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B867" s="5">
+        <v>101</v>
+      </c>
+      <c r="C867" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D867" s="8">
+        <v>4656.08</v>
+      </c>
+    </row>
+    <row r="868" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A868" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B868" s="5">
+        <v>101</v>
+      </c>
+      <c r="C868" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="D868" s="8">
+        <v>-639.84</v>
+      </c>
+    </row>
+    <row r="869" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A869" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B869" s="5">
+        <v>101</v>
+      </c>
+      <c r="C869" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D869" s="8">
+        <v>1848</v>
+      </c>
+    </row>
+    <row r="870" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A870" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B870" s="5">
+        <v>101</v>
+      </c>
+      <c r="C870" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D870" s="8">
+        <v>12354</v>
+      </c>
+    </row>
+    <row r="871" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A871" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B871" s="5">
+        <v>101</v>
+      </c>
+      <c r="C871" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D871" s="8">
+        <v>3432</v>
+      </c>
+    </row>
+    <row r="872" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A872" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B872" s="5">
+        <v>101</v>
+      </c>
+      <c r="C872" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D872" s="8">
+        <v>1137.79</v>
+      </c>
+    </row>
+    <row r="873" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A873" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B873" s="5">
+        <v>101</v>
+      </c>
+      <c r="C873" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D873" s="8">
+        <v>1899.2</v>
+      </c>
+    </row>
+    <row r="874" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A874" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B874" s="5">
+        <v>101</v>
+      </c>
+      <c r="C874" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D874" s="8">
+        <v>1899.2</v>
+      </c>
+    </row>
+    <row r="875" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A875" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B875" s="5">
+        <v>101</v>
+      </c>
+      <c r="C875" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D875" s="8">
+        <v>524.1</v>
+      </c>
+    </row>
+    <row r="876" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A876" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B876" s="5">
+        <v>101</v>
+      </c>
+      <c r="C876" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D876" s="8">
+        <v>1172.02</v>
+      </c>
+    </row>
+    <row r="877" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A877" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B877" s="5">
+        <v>101</v>
+      </c>
+      <c r="C877" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D877" s="8">
+        <v>9133.14</v>
+      </c>
+    </row>
+    <row r="878" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A878" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B878" s="5">
+        <v>101</v>
+      </c>
+      <c r="C878" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D878" s="8">
+        <v>1831.77</v>
+      </c>
+    </row>
+    <row r="879" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A879" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B879" s="5">
+        <v>101</v>
+      </c>
+      <c r="C879" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D879" s="8">
+        <v>25944.23</v>
+      </c>
+    </row>
+    <row r="880" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A880" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B880" s="5">
+        <v>101</v>
+      </c>
+      <c r="C880" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D880" s="8">
+        <v>104016.74</v>
+      </c>
+    </row>
+    <row r="881" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A881" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B881" s="5">
+        <v>101</v>
+      </c>
+      <c r="C881" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="D881" s="8">
+        <v>4432.3999999999996</v>
+      </c>
+    </row>
+    <row r="882" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A882" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B882" s="5">
+        <v>101</v>
+      </c>
+      <c r="C882" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="D882" s="8">
+        <v>1139.52</v>
+      </c>
+    </row>
+    <row r="883" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A883" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B883" s="5">
+        <v>101</v>
+      </c>
+      <c r="C883" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="D883" s="8">
+        <v>2859.4</v>
+      </c>
+    </row>
+    <row r="884" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A884" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B884" s="5">
+        <v>101</v>
+      </c>
+      <c r="C884" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D884" s="8">
+        <v>124297.77</v>
+      </c>
+    </row>
+    <row r="885" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A885" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B885" s="5">
+        <v>101</v>
+      </c>
+      <c r="C885" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="D885" s="8">
+        <v>-487.02</v>
+      </c>
+    </row>
+    <row r="886" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A886" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B886" s="5">
+        <v>101</v>
+      </c>
+      <c r="C886" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D886" s="8">
+        <v>26259.13</v>
+      </c>
+    </row>
+    <row r="887" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A887" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B887" s="5">
+        <v>101</v>
+      </c>
+      <c r="C887" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D887" s="8">
+        <v>305.2</v>
+      </c>
+    </row>
+    <row r="888" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A888" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B888" s="5">
+        <v>101</v>
+      </c>
+      <c r="C888" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D888" s="8">
+        <v>1481.55</v>
+      </c>
+    </row>
+    <row r="889" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A889" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B889" s="5">
+        <v>101</v>
+      </c>
+      <c r="C889" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D889" s="8">
+        <v>2326</v>
+      </c>
+    </row>
+    <row r="890" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A890" s="6">
+        <v>46321</v>
+      </c>
+      <c r="B890" s="5">
+        <v>101</v>
+      </c>
+      <c r="C890" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D890" s="8">
+        <v>1259.01</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização dos dados do faturamento
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F094D1D-294F-414B-BFEC-A1DEC515B7D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B69B647A-02C4-4198-A020-DF8034DAFEC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
   <sheets>
     <sheet name="FaturamentoBruto" sheetId="1" r:id="rId1"/>
@@ -1948,7 +1948,7 @@
         <v>46322</v>
       </c>
       <c r="B23">
-        <v>146303.18</v>
+        <v>333797.8</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -1959,7 +1959,7 @@
         <v>75</v>
       </c>
       <c r="B24" s="2">
-        <v>8845521.9800000004</v>
+        <v>9033016.5999999996</v>
       </c>
       <c r="C24" s="2">
         <v>-319379.15000000002</v>
@@ -2005,8 +2005,8 @@
     <hyperlink ref="C21" r:id="rId36" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{A5E30353-68AD-4555-A4A4-F43F7F15A167}"/>
     <hyperlink ref="B22" r:id="rId37" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F5D8DE54-95D1-46C8-88FE-0455E31F55EA}"/>
     <hyperlink ref="C22" r:id="rId38" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{B6508494-A2ED-45CE-A06F-52BAF7398889}"/>
-    <hyperlink ref="B23" r:id="rId39" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{E234A0FC-3F1D-4E49-89FE-CFF8150000F6}"/>
-    <hyperlink ref="C23" r:id="rId40" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{3AB773AA-3A9E-4C38-8792-28BC2A833A14}"/>
+    <hyperlink ref="B23" r:id="rId39" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{DD30AD69-0057-402B-A83E-B59DBD36F3B0}"/>
+    <hyperlink ref="C23" r:id="rId40" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{5B426AA7-E462-4457-8A68-E5B75510379A}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId41"/>

</xml_diff>

<commit_message>
Primeira atualização diária dos dados
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B69B647A-02C4-4198-A020-DF8034DAFEC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{665EC49B-C0C2-4D53-9B4D-E33D969C4799}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
   <sheets>
     <sheet name="FaturamentoBruto" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="246">
   <si>
     <t>Filial</t>
   </si>
@@ -747,6 +747,18 @@
   </si>
   <si>
     <t>DASA 61.486.650/0686</t>
+  </si>
+  <si>
+    <t>SOMA CAMPINAS 03.469</t>
+  </si>
+  <si>
+    <t>INSTITUTO HOC</t>
+  </si>
+  <si>
+    <t>HOSP DR. J M</t>
+  </si>
+  <si>
+    <t>GENERA SERVICOS LABO</t>
   </si>
 </sst>
 </file>
@@ -1948,10 +1960,10 @@
         <v>46322</v>
       </c>
       <c r="B23">
-        <v>333797.8</v>
+        <v>501074.18</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>-397.64</v>
       </c>
     </row>
     <row r="24" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
@@ -1959,10 +1971,10 @@
         <v>75</v>
       </c>
       <c r="B24" s="2">
-        <v>9033016.5999999996</v>
+        <v>9200292.9800000004</v>
       </c>
       <c r="C24" s="2">
-        <v>-319379.15000000002</v>
+        <v>-319776.78999999998</v>
       </c>
     </row>
   </sheetData>
@@ -2005,8 +2017,8 @@
     <hyperlink ref="C21" r:id="rId36" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{A5E30353-68AD-4555-A4A4-F43F7F15A167}"/>
     <hyperlink ref="B22" r:id="rId37" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F5D8DE54-95D1-46C8-88FE-0455E31F55EA}"/>
     <hyperlink ref="C22" r:id="rId38" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{B6508494-A2ED-45CE-A06F-52BAF7398889}"/>
-    <hyperlink ref="B23" r:id="rId39" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{DD30AD69-0057-402B-A83E-B59DBD36F3B0}"/>
-    <hyperlink ref="C23" r:id="rId40" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{5B426AA7-E462-4457-8A68-E5B75510379A}"/>
+    <hyperlink ref="B23" r:id="rId39" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{AEE793B7-F5AF-487A-B107-0E30AC64A5B3}"/>
+    <hyperlink ref="C23" r:id="rId40" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{5B2D560A-0C63-4359-ACFB-3F512F59B412}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId41"/>
@@ -2015,7 +2027,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2872C95-5BBD-470F-BA44-E40722CF8AA3}">
-  <dimension ref="A1:D890"/>
+  <dimension ref="A1:D948"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="5" bestFit="1" customWidth="1"/>
@@ -2026,17 +2038,17 @@
     <col min="6" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="4" t="s">
         <v>74</v>
       </c>
     </row>
@@ -14484,6 +14496,818 @@
       </c>
       <c r="D890" s="8">
         <v>1259.01</v>
+      </c>
+    </row>
+    <row r="891" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A891" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B891" s="5">
+        <v>101</v>
+      </c>
+      <c r="C891" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="D891" s="8">
+        <v>216925.18</v>
+      </c>
+    </row>
+    <row r="892" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A892" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B892" s="5">
+        <v>101</v>
+      </c>
+      <c r="C892" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="D892" s="8">
+        <v>13304.93</v>
+      </c>
+    </row>
+    <row r="893" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A893" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B893" s="5">
+        <v>101</v>
+      </c>
+      <c r="C893" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="D893" s="8">
+        <v>15819.99</v>
+      </c>
+    </row>
+    <row r="894" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A894" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B894" s="5">
+        <v>101</v>
+      </c>
+      <c r="C894" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="D894" s="8">
+        <v>186.3</v>
+      </c>
+    </row>
+    <row r="895" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A895" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B895" s="5">
+        <v>101</v>
+      </c>
+      <c r="C895" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D895" s="8">
+        <v>502.8</v>
+      </c>
+    </row>
+    <row r="896" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A896" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B896" s="5">
+        <v>101</v>
+      </c>
+      <c r="C896" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="D896" s="8">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="897" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A897" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B897" s="5">
+        <v>101</v>
+      </c>
+      <c r="C897" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D897" s="8">
+        <v>3207.44</v>
+      </c>
+    </row>
+    <row r="898" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A898" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B898" s="5">
+        <v>101</v>
+      </c>
+      <c r="C898" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D898" s="8">
+        <v>93.3</v>
+      </c>
+    </row>
+    <row r="899" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A899" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B899" s="5">
+        <v>101</v>
+      </c>
+      <c r="C899" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D899" s="8">
+        <v>174.02</v>
+      </c>
+    </row>
+    <row r="900" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A900" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B900" s="5">
+        <v>101</v>
+      </c>
+      <c r="C900" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="D900" s="8">
+        <v>1291.05</v>
+      </c>
+    </row>
+    <row r="901" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A901" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B901" s="5">
+        <v>101</v>
+      </c>
+      <c r="C901" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D901" s="8">
+        <v>-214.82</v>
+      </c>
+    </row>
+    <row r="902" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A902" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B902" s="5">
+        <v>101</v>
+      </c>
+      <c r="C902" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D902" s="8">
+        <v>5653</v>
+      </c>
+    </row>
+    <row r="903" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A903" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B903" s="5">
+        <v>101</v>
+      </c>
+      <c r="C903" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D903" s="8">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="904" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A904" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B904" s="5">
+        <v>101</v>
+      </c>
+      <c r="C904" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D904" s="8">
+        <v>566.6</v>
+      </c>
+    </row>
+    <row r="905" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A905" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B905" s="5">
+        <v>101</v>
+      </c>
+      <c r="C905" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="D905" s="8">
+        <v>50.7</v>
+      </c>
+    </row>
+    <row r="906" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A906" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B906" s="5">
+        <v>101</v>
+      </c>
+      <c r="C906" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D906" s="8">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="907" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A907" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B907" s="5">
+        <v>101</v>
+      </c>
+      <c r="C907" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D907" s="8">
+        <v>404.79</v>
+      </c>
+    </row>
+    <row r="908" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A908" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B908" s="5">
+        <v>101</v>
+      </c>
+      <c r="C908" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D908" s="8">
+        <v>252.69</v>
+      </c>
+    </row>
+    <row r="909" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A909" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B909" s="5">
+        <v>101</v>
+      </c>
+      <c r="C909" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D909" s="8">
+        <v>511.55</v>
+      </c>
+    </row>
+    <row r="910" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A910" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B910" s="5">
+        <v>101</v>
+      </c>
+      <c r="C910" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="D910" s="8">
+        <v>651.20000000000005</v>
+      </c>
+    </row>
+    <row r="911" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A911" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B911" s="5">
+        <v>101</v>
+      </c>
+      <c r="C911" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D911" s="8">
+        <v>1905.73</v>
+      </c>
+    </row>
+    <row r="912" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A912" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B912" s="5">
+        <v>101</v>
+      </c>
+      <c r="C912" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D912" s="8">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="913" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A913" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B913" s="5">
+        <v>101</v>
+      </c>
+      <c r="C913" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D913" s="8">
+        <v>24812.44</v>
+      </c>
+    </row>
+    <row r="914" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A914" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B914" s="5">
+        <v>101</v>
+      </c>
+      <c r="C914" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="D914" s="8">
+        <v>65.680000000000007</v>
+      </c>
+    </row>
+    <row r="915" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A915" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B915" s="5">
+        <v>101</v>
+      </c>
+      <c r="C915" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D915" s="8">
+        <v>17556.349999999999</v>
+      </c>
+    </row>
+    <row r="916" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A916" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B916" s="5">
+        <v>101</v>
+      </c>
+      <c r="C916" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D916" s="8">
+        <v>3969.77</v>
+      </c>
+    </row>
+    <row r="917" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A917" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B917" s="5">
+        <v>101</v>
+      </c>
+      <c r="C917" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D917" s="8">
+        <v>1683</v>
+      </c>
+    </row>
+    <row r="918" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A918" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B918" s="5">
+        <v>101</v>
+      </c>
+      <c r="C918" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="D918" s="8">
+        <v>845.5</v>
+      </c>
+    </row>
+    <row r="919" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A919" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B919" s="5">
+        <v>101</v>
+      </c>
+      <c r="C919" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="D919" s="8">
+        <v>116091.37</v>
+      </c>
+    </row>
+    <row r="920" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A920" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B920" s="5">
+        <v>101</v>
+      </c>
+      <c r="C920" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D920" s="8">
+        <v>2558.52</v>
+      </c>
+    </row>
+    <row r="921" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A921" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B921" s="5">
+        <v>101</v>
+      </c>
+      <c r="C921" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="D921" s="8">
+        <v>1403.02</v>
+      </c>
+    </row>
+    <row r="922" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A922" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B922" s="5">
+        <v>101</v>
+      </c>
+      <c r="C922" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D922" s="8">
+        <v>593.46</v>
+      </c>
+    </row>
+    <row r="923" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A923" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B923" s="5">
+        <v>101</v>
+      </c>
+      <c r="C923" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D923" s="8">
+        <v>1227.48</v>
+      </c>
+    </row>
+    <row r="924" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A924" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B924" s="5">
+        <v>101</v>
+      </c>
+      <c r="C924" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D924" s="8">
+        <v>1979.94</v>
+      </c>
+    </row>
+    <row r="925" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A925" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B925" s="5">
+        <v>101</v>
+      </c>
+      <c r="C925" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D925" s="8">
+        <v>3696</v>
+      </c>
+    </row>
+    <row r="926" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A926" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B926" s="5">
+        <v>101</v>
+      </c>
+      <c r="C926" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D926" s="8">
+        <v>7054.3</v>
+      </c>
+    </row>
+    <row r="927" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A927" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B927" s="5">
+        <v>101</v>
+      </c>
+      <c r="C927" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D927" s="8">
+        <v>4382.76</v>
+      </c>
+    </row>
+    <row r="928" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A928" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B928" s="5">
+        <v>101</v>
+      </c>
+      <c r="C928" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D928" s="8">
+        <v>1867.78</v>
+      </c>
+    </row>
+    <row r="929" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A929" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B929" s="5">
+        <v>101</v>
+      </c>
+      <c r="C929" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D929" s="8">
+        <v>687.8</v>
+      </c>
+    </row>
+    <row r="930" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A930" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B930" s="5">
+        <v>101</v>
+      </c>
+      <c r="C930" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D930" s="8">
+        <v>11332</v>
+      </c>
+    </row>
+    <row r="931" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A931" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B931" s="5">
+        <v>101</v>
+      </c>
+      <c r="C931" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D931" s="8">
+        <v>3461.43</v>
+      </c>
+    </row>
+    <row r="932" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A932" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B932" s="5">
+        <v>101</v>
+      </c>
+      <c r="C932" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D932" s="8">
+        <v>75.760000000000005</v>
+      </c>
+    </row>
+    <row r="933" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A933" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B933" s="5">
+        <v>101</v>
+      </c>
+      <c r="C933" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D933" s="8">
+        <v>52.03</v>
+      </c>
+    </row>
+    <row r="934" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A934" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B934" s="5">
+        <v>101</v>
+      </c>
+      <c r="C934" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D934" s="8">
+        <v>433.1</v>
+      </c>
+    </row>
+    <row r="935" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A935" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B935" s="5">
+        <v>101</v>
+      </c>
+      <c r="C935" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D935" s="8">
+        <v>163.85</v>
+      </c>
+    </row>
+    <row r="936" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A936" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B936" s="5">
+        <v>101</v>
+      </c>
+      <c r="C936" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D936" s="8">
+        <v>8030.12</v>
+      </c>
+    </row>
+    <row r="937" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A937" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B937" s="5">
+        <v>101</v>
+      </c>
+      <c r="C937" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="D937" s="8">
+        <v>763.47</v>
+      </c>
+    </row>
+    <row r="938" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A938" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B938" s="5">
+        <v>101</v>
+      </c>
+      <c r="C938" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="D938" s="8">
+        <v>4705.68</v>
+      </c>
+    </row>
+    <row r="939" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A939" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B939" s="5">
+        <v>101</v>
+      </c>
+      <c r="C939" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D939" s="8">
+        <v>1272.45</v>
+      </c>
+    </row>
+    <row r="940" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A940" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B940" s="5">
+        <v>101</v>
+      </c>
+      <c r="C940" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D940" s="8">
+        <v>10687</v>
+      </c>
+    </row>
+    <row r="941" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A941" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B941" s="5">
+        <v>101</v>
+      </c>
+      <c r="C941" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D941" s="8">
+        <v>21714</v>
+      </c>
+    </row>
+    <row r="942" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A942" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B942" s="5">
+        <v>101</v>
+      </c>
+      <c r="C942" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="D942" s="8">
+        <v>-182.82</v>
+      </c>
+    </row>
+    <row r="943" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A943" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B943" s="5">
+        <v>101</v>
+      </c>
+      <c r="C943" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D943" s="8">
+        <v>1815.66</v>
+      </c>
+    </row>
+    <row r="944" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A944" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B944" s="5">
+        <v>101</v>
+      </c>
+      <c r="C944" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D944" s="8">
+        <v>988.45</v>
+      </c>
+    </row>
+    <row r="945" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A945" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B945" s="5">
+        <v>101</v>
+      </c>
+      <c r="C945" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D945" s="8">
+        <v>821.8</v>
+      </c>
+    </row>
+    <row r="946" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A946" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B946" s="5">
+        <v>101</v>
+      </c>
+      <c r="C946" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D946" s="8">
+        <v>610.4</v>
+      </c>
+    </row>
+    <row r="947" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A947" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B947" s="5">
+        <v>101</v>
+      </c>
+      <c r="C947" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D947" s="8">
+        <v>3412.9</v>
+      </c>
+    </row>
+    <row r="948" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A948" s="6">
+        <v>46322</v>
+      </c>
+      <c r="B948" s="5">
+        <v>101</v>
+      </c>
+      <c r="C948" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D948" s="8">
+        <v>213.64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Final da atualização diária dos dados
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{665EC49B-C0C2-4D53-9B4D-E33D969C4799}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1711666A-997D-4D0B-9B08-1367F1DAB6D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
   <sheets>
     <sheet name="FaturamentoBruto" sheetId="1" r:id="rId1"/>
@@ -1711,7 +1711,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19101EBF-008C-4E37-90C0-CF2D419D5300}">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15.75" thickBottom="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="3" bestFit="1" customWidth="1"/>
@@ -1967,14 +1967,25 @@
       </c>
     </row>
     <row r="24" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="3">
+        <v>46323</v>
+      </c>
+      <c r="B24">
+        <v>346987.98</v>
+      </c>
+      <c r="C24">
+        <v>-14081.69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B24" s="2">
-        <v>9200292.9800000004</v>
-      </c>
-      <c r="C24" s="2">
-        <v>-319776.78999999998</v>
+      <c r="B25" s="2">
+        <v>9449348.9600000009</v>
+      </c>
+      <c r="C25" s="2">
+        <v>-333858.48</v>
       </c>
     </row>
   </sheetData>
@@ -2019,9 +2030,11 @@
     <hyperlink ref="C22" r:id="rId38" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{B6508494-A2ED-45CE-A06F-52BAF7398889}"/>
     <hyperlink ref="B23" r:id="rId39" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{AEE793B7-F5AF-487A-B107-0E30AC64A5B3}"/>
     <hyperlink ref="C23" r:id="rId40" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{5B2D560A-0C63-4359-ACFB-3F512F59B412}"/>
+    <hyperlink ref="B24" r:id="rId41" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{AFF04227-3C77-4389-88C6-89725CA803DA}"/>
+    <hyperlink ref="C24" r:id="rId42" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{123386E2-900D-431C-A53B-090E37DD1B5B}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId41"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId43"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: Primeira atualização diária dos dados
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1711666A-997D-4D0B-9B08-1367F1DAB6D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34E9EC6B-862D-4F8B-BC67-0222A14F6142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
   <sheets>
     <sheet name="FaturamentoBruto" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1003" uniqueCount="248">
   <si>
     <t>Filial</t>
   </si>
@@ -759,6 +759,12 @@
   </si>
   <si>
     <t>GENERA SERVICOS LABO</t>
+  </si>
+  <si>
+    <t>MEDISE</t>
+  </si>
+  <si>
+    <t>CONGREGACAO</t>
   </si>
 </sst>
 </file>
@@ -1107,7 +1113,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -1267,6 +1273,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDEE2E6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1312,7 +1333,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1335,6 +1356,9 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="19" fillId="33" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1967,11 +1991,11 @@
       </c>
     </row>
     <row r="24" spans="1:3" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="3">
+      <c r="A24" s="9">
         <v>46323</v>
       </c>
       <c r="B24">
-        <v>346987.98</v>
+        <v>367755.97</v>
       </c>
       <c r="C24">
         <v>-14081.69</v>
@@ -1982,7 +2006,7 @@
         <v>75</v>
       </c>
       <c r="B25" s="2">
-        <v>9449348.9600000009</v>
+        <v>9470116.9499999993</v>
       </c>
       <c r="C25" s="2">
         <v>-333858.48</v>
@@ -2030,8 +2054,8 @@
     <hyperlink ref="C22" r:id="rId38" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{B6508494-A2ED-45CE-A06F-52BAF7398889}"/>
     <hyperlink ref="B23" r:id="rId39" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{AEE793B7-F5AF-487A-B107-0E30AC64A5B3}"/>
     <hyperlink ref="C23" r:id="rId40" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{5B2D560A-0C63-4359-ACFB-3F512F59B412}"/>
-    <hyperlink ref="B24" r:id="rId41" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{AFF04227-3C77-4389-88C6-89725CA803DA}"/>
-    <hyperlink ref="C24" r:id="rId42" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{123386E2-900D-431C-A53B-090E37DD1B5B}"/>
+    <hyperlink ref="B24" r:id="rId41" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{34D1B18E-35BC-42C7-9732-5F6E5B4D5F23}"/>
+    <hyperlink ref="C24" r:id="rId42" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{76B454AD-05EE-48D8-8898-81B3D35B99AC}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId43"/>
@@ -2040,15 +2064,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2872C95-5BBD-470F-BA44-E40722CF8AA3}">
-  <dimension ref="A1:D948"/>
+  <dimension ref="A1:D995"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.28515625" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.5703125" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="5"/>
+    <col min="5" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -15323,6 +15346,664 @@
         <v>213.64</v>
       </c>
     </row>
+    <row r="949" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A949" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B949" s="5">
+        <v>101</v>
+      </c>
+      <c r="C949" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="D949" s="8">
+        <v>117397.42</v>
+      </c>
+    </row>
+    <row r="950" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A950" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B950" s="5">
+        <v>101</v>
+      </c>
+      <c r="C950" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D950" s="8">
+        <v>12117.82</v>
+      </c>
+    </row>
+    <row r="951" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A951" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B951" s="5">
+        <v>101</v>
+      </c>
+      <c r="C951" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D951" s="8">
+        <v>12102.4</v>
+      </c>
+    </row>
+    <row r="952" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A952" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B952" s="5">
+        <v>101</v>
+      </c>
+      <c r="C952" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D952" s="5">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="953" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A953" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B953" s="5">
+        <v>101</v>
+      </c>
+      <c r="C953" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D953" s="8">
+        <v>1213.28</v>
+      </c>
+    </row>
+    <row r="954" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A954" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B954" s="5">
+        <v>101</v>
+      </c>
+      <c r="C954" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="D954" s="8">
+        <v>4620</v>
+      </c>
+    </row>
+    <row r="955" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A955" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B955" s="5">
+        <v>101</v>
+      </c>
+      <c r="C955" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D955" s="5">
+        <v>-642.34</v>
+      </c>
+    </row>
+    <row r="956" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A956" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B956" s="5">
+        <v>101</v>
+      </c>
+      <c r="C956" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D956" s="8">
+        <v>-4746.6000000000004</v>
+      </c>
+    </row>
+    <row r="957" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A957" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B957" s="5">
+        <v>101</v>
+      </c>
+      <c r="C957" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D957" s="8">
+        <v>23280</v>
+      </c>
+    </row>
+    <row r="958" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A958" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B958" s="5">
+        <v>101</v>
+      </c>
+      <c r="C958" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="D958" s="8">
+        <v>10841.95</v>
+      </c>
+    </row>
+    <row r="959" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A959" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B959" s="5">
+        <v>101</v>
+      </c>
+      <c r="C959" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D959" s="8">
+        <v>-1036</v>
+      </c>
+    </row>
+    <row r="960" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A960" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B960" s="5">
+        <v>101</v>
+      </c>
+      <c r="C960" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D960" s="8">
+        <v>2924.4</v>
+      </c>
+    </row>
+    <row r="961" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A961" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B961" s="5">
+        <v>101</v>
+      </c>
+      <c r="C961" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D961" s="8">
+        <v>15505.63</v>
+      </c>
+    </row>
+    <row r="962" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A962" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B962" s="5">
+        <v>101</v>
+      </c>
+      <c r="C962" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="D962" s="8">
+        <v>9934.01</v>
+      </c>
+    </row>
+    <row r="963" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A963" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B963" s="5">
+        <v>101</v>
+      </c>
+      <c r="C963" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D963" s="8">
+        <v>1337.85</v>
+      </c>
+    </row>
+    <row r="964" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A964" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B964" s="5">
+        <v>101</v>
+      </c>
+      <c r="C964" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D964" s="8">
+        <v>40166.03</v>
+      </c>
+    </row>
+    <row r="965" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A965" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B965" s="5">
+        <v>101</v>
+      </c>
+      <c r="C965" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D965" s="8">
+        <v>1583</v>
+      </c>
+    </row>
+    <row r="966" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A966" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B966" s="5">
+        <v>101</v>
+      </c>
+      <c r="C966" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D966" s="8">
+        <v>28889.22</v>
+      </c>
+    </row>
+    <row r="967" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A967" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B967" s="5">
+        <v>101</v>
+      </c>
+      <c r="C967" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D967" s="8">
+        <v>-2797.2</v>
+      </c>
+    </row>
+    <row r="968" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A968" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B968" s="5">
+        <v>101</v>
+      </c>
+      <c r="C968" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D968" s="8">
+        <v>7270.12</v>
+      </c>
+    </row>
+    <row r="969" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A969" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B969" s="5">
+        <v>101</v>
+      </c>
+      <c r="C969" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D969" s="8">
+        <v>1899.2</v>
+      </c>
+    </row>
+    <row r="970" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A970" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B970" s="5">
+        <v>101</v>
+      </c>
+      <c r="C970" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D970" s="8">
+        <v>11332</v>
+      </c>
+    </row>
+    <row r="971" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A971" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B971" s="5">
+        <v>101</v>
+      </c>
+      <c r="C971" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D971" s="8">
+        <v>3154.98</v>
+      </c>
+    </row>
+    <row r="972" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A972" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B972" s="5">
+        <v>101</v>
+      </c>
+      <c r="C972" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D972" s="8">
+        <v>4590.1400000000003</v>
+      </c>
+    </row>
+    <row r="973" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A973" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B973" s="5">
+        <v>101</v>
+      </c>
+      <c r="C973" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D973" s="8">
+        <v>8741.0300000000007</v>
+      </c>
+    </row>
+    <row r="974" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A974" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B974" s="5">
+        <v>101</v>
+      </c>
+      <c r="C974" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D974" s="5">
+        <v>416.9</v>
+      </c>
+    </row>
+    <row r="975" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A975" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B975" s="5">
+        <v>101</v>
+      </c>
+      <c r="C975" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D975" s="8">
+        <v>1023.65</v>
+      </c>
+    </row>
+    <row r="976" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A976" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B976" s="5">
+        <v>101</v>
+      </c>
+      <c r="C976" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D976" s="8">
+        <v>4587.47</v>
+      </c>
+    </row>
+    <row r="977" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A977" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B977" s="5">
+        <v>101</v>
+      </c>
+      <c r="C977" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D977" s="8">
+        <v>1990.08</v>
+      </c>
+    </row>
+    <row r="978" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A978" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B978" s="5">
+        <v>101</v>
+      </c>
+      <c r="C978" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D978" s="8">
+        <v>2023.32</v>
+      </c>
+    </row>
+    <row r="979" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A979" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B979" s="5">
+        <v>101</v>
+      </c>
+      <c r="C979" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="D979" s="8">
+        <v>2760</v>
+      </c>
+    </row>
+    <row r="980" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A980" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B980" s="5">
+        <v>101</v>
+      </c>
+      <c r="C980" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="D980" s="5">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="981" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A981" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B981" s="5">
+        <v>101</v>
+      </c>
+      <c r="C981" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D981" s="5">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="982" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A982" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B982" s="5">
+        <v>101</v>
+      </c>
+      <c r="C982" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D982" s="8">
+        <v>27847.200000000001</v>
+      </c>
+    </row>
+    <row r="983" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A983" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B983" s="5">
+        <v>101</v>
+      </c>
+      <c r="C983" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="D983" s="8">
+        <v>-4320</v>
+      </c>
+    </row>
+    <row r="984" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A984" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B984" s="5">
+        <v>101</v>
+      </c>
+      <c r="C984" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D984" s="8">
+        <v>1067.04</v>
+      </c>
+    </row>
+    <row r="985" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A985" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B985" s="5">
+        <v>101</v>
+      </c>
+      <c r="C985" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D985" s="5">
+        <v>608.28</v>
+      </c>
+    </row>
+    <row r="986" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A986" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B986" s="5">
+        <v>101</v>
+      </c>
+      <c r="C986" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D986" s="8">
+        <v>1689.5</v>
+      </c>
+    </row>
+    <row r="987" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A987" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B987" s="5">
+        <v>101</v>
+      </c>
+      <c r="C987" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D987" s="5">
+        <v>710.41</v>
+      </c>
+    </row>
+    <row r="988" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A988" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B988" s="5">
+        <v>101</v>
+      </c>
+      <c r="C988" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D988" s="5">
+        <v>457.8</v>
+      </c>
+    </row>
+    <row r="989" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A989" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B989" s="5">
+        <v>101</v>
+      </c>
+      <c r="C989" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D989" s="5">
+        <v>-539.54999999999995</v>
+      </c>
+    </row>
+    <row r="990" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A990" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B990" s="5">
+        <v>101</v>
+      </c>
+      <c r="C990" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D990" s="5">
+        <v>457.8</v>
+      </c>
+    </row>
+    <row r="991" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A991" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B991" s="5">
+        <v>101</v>
+      </c>
+      <c r="C991" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D991" s="5">
+        <v>373.9</v>
+      </c>
+    </row>
+    <row r="992" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A992" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B992" s="5">
+        <v>101</v>
+      </c>
+      <c r="C992" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D992" s="5">
+        <v>366.24</v>
+      </c>
+    </row>
+    <row r="993" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A993" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B993" s="5">
+        <v>101</v>
+      </c>
+      <c r="C993" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D993" s="5">
+        <v>396.76</v>
+      </c>
+    </row>
+    <row r="994" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A994" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B994" s="5">
+        <v>101</v>
+      </c>
+      <c r="C994" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D994" s="5">
+        <v>224.34</v>
+      </c>
+    </row>
+    <row r="995" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A995" s="6">
+        <v>46323</v>
+      </c>
+      <c r="B995" s="5">
+        <v>101</v>
+      </c>
+      <c r="C995" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="D995" s="5">
+        <v>100.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: correção no campo de faturamento
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C9E092-B214-420C-9E40-CD84F2C211ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A4FC15-C52A-4F70-9FBF-C90ABE967B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
@@ -2521,7 +2521,7 @@
         <v>0</v>
       </c>
       <c r="J26" s="9">
-        <v>0</v>
+        <v>9789630.4499999993</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Correção no problema do faturamento, mudança de lugar dos KPIs e novo KPI de devolução e média de devolução
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0A4FC15-C52A-4F70-9FBF-C90ABE967B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47D6FC34-69BE-420C-B4F6-814AC15640A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1036" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="252">
   <si>
     <t>Filial</t>
   </si>
@@ -777,34 +777,13 @@
   </si>
   <si>
     <t>TOT</t>
-  </si>
-  <si>
-    <t>qui</t>
-  </si>
-  <si>
-    <t>sex</t>
-  </si>
-  <si>
-    <t>seg</t>
-  </si>
-  <si>
-    <t>ter</t>
-  </si>
-  <si>
-    <t>qua</t>
-  </si>
-  <si>
-    <t>sáb</t>
-  </si>
-  <si>
-    <t>dom</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -951,6 +930,29 @@
       <color rgb="FF212529"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.6"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.6"/>
+      <color rgb="FF212529"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="35">
@@ -1146,7 +1148,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -1293,15 +1295,54 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="FFDEE2E6"/>
+        <color rgb="FF808080"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
       </left>
       <right style="medium">
-        <color rgb="FFDEE2E6"/>
+        <color rgb="FF808080"/>
       </right>
       <top style="medium">
-        <color rgb="FFDEE2E6"/>
+        <color rgb="FF808080"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FF808080"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1309,9 +1350,11 @@
         <color rgb="FFDEE2E6"/>
       </left>
       <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
         <color rgb="FFDEE2E6"/>
-      </right>
-      <top/>
+      </top>
       <bottom style="medium">
         <color rgb="FFDEE2E6"/>
       </bottom>
@@ -1319,15 +1362,21 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="FFDEE2E6"/>
+        <color rgb="FF808080"/>
       </left>
-      <right/>
-      <top/>
-      <bottom/>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -1370,8 +1419,9 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="19" fillId="33" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1389,21 +1439,53 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="19" fillId="33" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="22" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="19" fillId="33" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="4" fontId="20" fillId="0" borderId="11" xfId="42" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" xfId="42" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="4" fontId="22" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="21" fillId="34" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Ênfase2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Ênfase3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -1433,6 +1515,7 @@
     <cellStyle name="Ênfase5" xfId="34" builtinId="45" customBuiltin="1"/>
     <cellStyle name="Ênfase6" xfId="38" builtinId="49" customBuiltin="1"/>
     <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Hiperlink" xfId="42" builtinId="8"/>
     <cellStyle name="Neutro" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Nota" xfId="15" builtinId="10" customBuiltin="1"/>
@@ -1781,758 +1864,879 @@
   <sheetFormatPr defaultRowHeight="15.75" thickBottom="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.140625" customWidth="1"/>
-    <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10" t="s">
+      <c r="E1" s="19"/>
+      <c r="F1" s="18" t="s">
         <v>249</v>
       </c>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10" t="s">
+      <c r="G1" s="19"/>
+      <c r="H1" s="18" t="s">
         <v>250</v>
       </c>
-      <c r="I1" s="10"/>
-    </row>
-    <row r="2" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="8"/>
-      <c r="B2" t="s">
+      <c r="I1" s="19"/>
+      <c r="J1" s="20" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="17"/>
+      <c r="B2" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="J2" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="B3" s="5">
+      <c r="J2" s="21"/>
+    </row>
+    <row r="3" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
         <v>46296</v>
       </c>
-      <c r="C3" s="9">
+      <c r="B3" s="10">
         <v>271426.78000000003</v>
       </c>
-      <c r="D3">
+      <c r="C3" s="11">
         <v>0</v>
       </c>
-      <c r="E3">
+      <c r="D3" s="11">
         <v>619.79999999999995</v>
       </c>
-      <c r="F3">
+      <c r="E3" s="11">
         <v>0</v>
       </c>
-      <c r="H3">
+      <c r="F3" s="8"/>
+      <c r="G3" s="11">
         <v>0</v>
       </c>
-      <c r="I3">
+      <c r="H3" s="8"/>
+      <c r="I3" s="11">
         <v>0</v>
       </c>
-      <c r="J3" s="9">
+      <c r="J3" s="12">
         <v>272046.58</v>
       </c>
     </row>
     <row r="4" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="B4" s="5">
+      <c r="A4" s="9">
         <v>46297</v>
       </c>
-      <c r="C4" s="9">
+      <c r="B4" s="10">
         <v>423201.75</v>
       </c>
-      <c r="D4" s="9">
+      <c r="C4" s="10">
         <v>-26599.88</v>
       </c>
-      <c r="E4" s="9">
+      <c r="D4" s="10">
         <v>60744.65</v>
       </c>
-      <c r="F4">
+      <c r="E4" s="11">
         <v>0</v>
       </c>
-      <c r="H4">
+      <c r="F4" s="8"/>
+      <c r="G4" s="11">
         <v>0</v>
       </c>
-      <c r="I4">
+      <c r="H4" s="8"/>
+      <c r="I4" s="11">
         <v>0</v>
       </c>
-      <c r="J4" s="9">
+      <c r="J4" s="12">
         <v>457346.52</v>
       </c>
     </row>
     <row r="5" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="B5" s="5">
+      <c r="A5" s="9">
         <v>46300</v>
       </c>
-      <c r="C5" s="9">
+      <c r="B5" s="10">
         <v>279190.96000000002</v>
       </c>
-      <c r="D5" s="9">
+      <c r="C5" s="10">
         <v>-7502.05</v>
       </c>
-      <c r="E5" s="9">
+      <c r="D5" s="10">
         <v>33687.550000000003</v>
       </c>
-      <c r="F5">
+      <c r="E5" s="11">
         <v>0</v>
       </c>
-      <c r="H5">
+      <c r="F5" s="8"/>
+      <c r="G5" s="11">
         <v>0</v>
       </c>
-      <c r="I5">
+      <c r="H5" s="8"/>
+      <c r="I5" s="11">
         <v>0</v>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="12">
         <v>305376.46000000002</v>
       </c>
     </row>
     <row r="6" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="B6" s="5">
+      <c r="A6" s="9">
         <v>46301</v>
       </c>
-      <c r="C6" s="9">
+      <c r="B6" s="10">
         <v>425539.17</v>
       </c>
-      <c r="D6" s="9">
+      <c r="C6" s="10">
         <v>-15443.4</v>
       </c>
-      <c r="E6" s="9">
+      <c r="D6" s="10">
         <v>51272.05</v>
       </c>
-      <c r="F6">
+      <c r="E6" s="11">
         <v>-149.56</v>
       </c>
-      <c r="H6">
+      <c r="F6" s="8"/>
+      <c r="G6" s="11">
         <v>0</v>
       </c>
-      <c r="I6">
+      <c r="H6" s="8"/>
+      <c r="I6" s="11">
         <v>0</v>
       </c>
-      <c r="J6" s="9">
+      <c r="J6" s="12">
         <v>461218.26</v>
       </c>
     </row>
     <row r="7" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="B7" s="5">
+      <c r="A7" s="9">
         <v>46302</v>
       </c>
-      <c r="C7" s="9">
+      <c r="B7" s="10">
         <v>306641.53000000003</v>
       </c>
-      <c r="D7" s="9">
+      <c r="C7" s="10">
         <v>-12949.2</v>
       </c>
-      <c r="E7" s="9">
+      <c r="D7" s="10">
         <v>26119.68</v>
       </c>
-      <c r="F7">
+      <c r="E7" s="11">
         <v>0</v>
       </c>
-      <c r="H7">
+      <c r="F7" s="8"/>
+      <c r="G7" s="11">
         <v>0</v>
       </c>
-      <c r="I7">
+      <c r="H7" s="8"/>
+      <c r="I7" s="11">
         <v>0</v>
       </c>
-      <c r="J7" s="9">
+      <c r="J7" s="12">
         <v>319812.01</v>
       </c>
     </row>
     <row r="8" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="B8" s="5">
+      <c r="A8" s="9">
         <v>46303</v>
       </c>
-      <c r="C8" s="9">
+      <c r="B8" s="10">
         <v>578381.43999999994</v>
       </c>
-      <c r="D8">
+      <c r="C8" s="11">
         <v>0</v>
       </c>
-      <c r="E8" s="9">
+      <c r="D8" s="10">
         <v>14425.52</v>
       </c>
-      <c r="F8">
+      <c r="E8" s="11">
         <v>0</v>
       </c>
-      <c r="H8">
+      <c r="F8" s="8"/>
+      <c r="G8" s="11">
         <v>0</v>
       </c>
-      <c r="I8">
+      <c r="H8" s="8"/>
+      <c r="I8" s="11">
         <v>0</v>
       </c>
-      <c r="J8" s="9">
+      <c r="J8" s="12">
         <v>592806.96</v>
       </c>
     </row>
     <row r="9" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="B9" s="5">
+      <c r="A9" s="9">
         <v>46304</v>
       </c>
-      <c r="C9" s="9">
+      <c r="B9" s="10">
         <v>307842.78999999998</v>
       </c>
-      <c r="D9" s="9">
+      <c r="C9" s="10">
         <v>-70366.45</v>
       </c>
-      <c r="E9" s="9">
+      <c r="D9" s="10">
         <v>46378.81</v>
       </c>
-      <c r="F9">
+      <c r="E9" s="11">
         <v>-317</v>
       </c>
-      <c r="H9">
+      <c r="F9" s="8"/>
+      <c r="G9" s="11">
         <v>0</v>
       </c>
-      <c r="I9">
+      <c r="H9" s="8"/>
+      <c r="I9" s="11">
         <v>0</v>
       </c>
-      <c r="J9" s="9">
+      <c r="J9" s="12">
         <v>283538.15000000002</v>
       </c>
     </row>
     <row r="10" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="B10" s="5">
+      <c r="A10" s="9">
         <v>46305</v>
       </c>
-      <c r="C10" s="9">
+      <c r="B10" s="10">
         <v>203772.98</v>
       </c>
-      <c r="D10">
+      <c r="C10" s="11">
         <v>0</v>
       </c>
-      <c r="F10">
+      <c r="D10" s="8"/>
+      <c r="E10" s="11">
         <v>0</v>
       </c>
-      <c r="H10">
+      <c r="F10" s="8"/>
+      <c r="G10" s="11">
         <v>0</v>
       </c>
-      <c r="I10">
+      <c r="H10" s="8"/>
+      <c r="I10" s="11">
         <v>0</v>
       </c>
-      <c r="J10" s="9">
+      <c r="J10" s="12">
         <v>203772.98</v>
       </c>
     </row>
     <row r="11" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="B11" s="5">
+      <c r="A11" s="9">
         <v>46306</v>
       </c>
-      <c r="C11" s="9">
+      <c r="B11" s="10">
         <v>169560.7</v>
       </c>
-      <c r="D11">
+      <c r="C11" s="11">
         <v>0</v>
       </c>
-      <c r="F11">
+      <c r="D11" s="8"/>
+      <c r="E11" s="11">
         <v>0</v>
       </c>
-      <c r="H11">
+      <c r="F11" s="8"/>
+      <c r="G11" s="11">
         <v>0</v>
       </c>
-      <c r="I11">
+      <c r="H11" s="8"/>
+      <c r="I11" s="11">
         <v>0</v>
       </c>
-      <c r="J11" s="9">
+      <c r="J11" s="12">
         <v>169560.7</v>
       </c>
     </row>
     <row r="12" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="B12" s="5">
+      <c r="A12" s="9">
         <v>46307</v>
       </c>
-      <c r="C12" s="9">
+      <c r="B12" s="10">
         <v>216275.07</v>
       </c>
-      <c r="D12">
+      <c r="C12" s="11">
         <v>0</v>
       </c>
-      <c r="F12">
+      <c r="D12" s="8"/>
+      <c r="E12" s="11">
         <v>0</v>
       </c>
-      <c r="H12">
+      <c r="F12" s="8"/>
+      <c r="G12" s="11">
         <v>0</v>
       </c>
-      <c r="I12">
+      <c r="H12" s="8"/>
+      <c r="I12" s="11">
         <v>0</v>
       </c>
-      <c r="J12" s="9">
+      <c r="J12" s="12">
         <v>216275.07</v>
       </c>
     </row>
     <row r="13" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="B13" s="5">
+      <c r="A13" s="9">
         <v>46308</v>
       </c>
-      <c r="C13" s="9">
+      <c r="B13" s="10">
         <v>476395.59</v>
       </c>
-      <c r="D13" s="9">
+      <c r="C13" s="10">
         <v>-29468.28</v>
       </c>
-      <c r="E13" s="9">
+      <c r="D13" s="10">
         <v>57788.11</v>
       </c>
-      <c r="F13">
+      <c r="E13" s="11">
         <v>0</v>
       </c>
-      <c r="H13">
+      <c r="F13" s="8"/>
+      <c r="G13" s="11">
         <v>0</v>
       </c>
-      <c r="I13">
+      <c r="H13" s="8"/>
+      <c r="I13" s="11">
         <v>0</v>
       </c>
-      <c r="J13" s="9">
+      <c r="J13" s="12">
         <v>504715.42</v>
       </c>
     </row>
     <row r="14" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="B14" s="5">
+      <c r="A14" s="9">
         <v>46309</v>
       </c>
-      <c r="C14" s="9">
+      <c r="B14" s="10">
         <v>278778.15999999997</v>
       </c>
-      <c r="D14" s="9">
+      <c r="C14" s="10">
         <v>-14134.51</v>
       </c>
-      <c r="E14" s="9">
+      <c r="D14" s="10">
         <v>70986.45</v>
       </c>
-      <c r="F14">
+      <c r="E14" s="11">
         <v>0</v>
       </c>
-      <c r="H14">
+      <c r="F14" s="8"/>
+      <c r="G14" s="11">
         <v>0</v>
       </c>
-      <c r="I14">
+      <c r="H14" s="8"/>
+      <c r="I14" s="11">
         <v>0</v>
       </c>
-      <c r="J14" s="9">
+      <c r="J14" s="12">
         <v>335630.1</v>
       </c>
     </row>
     <row r="15" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="B15" s="5">
+      <c r="A15" s="9">
         <v>46310</v>
       </c>
-      <c r="C15" s="9">
+      <c r="B15" s="10">
         <v>281419.15999999997</v>
       </c>
-      <c r="D15">
+      <c r="C15" s="11">
         <v>0</v>
       </c>
-      <c r="E15" s="9">
+      <c r="D15" s="10">
         <v>33803.629999999997</v>
       </c>
-      <c r="F15" s="9">
+      <c r="E15" s="10">
         <v>-11085.38</v>
       </c>
-      <c r="H15">
+      <c r="F15" s="8"/>
+      <c r="G15" s="11">
         <v>0</v>
       </c>
-      <c r="I15">
+      <c r="H15" s="8"/>
+      <c r="I15" s="11">
         <v>0</v>
       </c>
-      <c r="J15" s="9">
+      <c r="J15" s="12">
         <v>304137.40999999997</v>
       </c>
     </row>
     <row r="16" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="B16" s="5">
+      <c r="A16" s="9">
         <v>46311</v>
       </c>
-      <c r="C16" s="9">
+      <c r="B16" s="10">
         <v>1353057.37</v>
       </c>
-      <c r="D16">
+      <c r="C16" s="11">
         <v>0</v>
       </c>
-      <c r="E16" s="9">
+      <c r="D16" s="10">
         <v>29492.51</v>
       </c>
-      <c r="F16">
+      <c r="E16" s="11">
         <v>0</v>
       </c>
-      <c r="H16">
+      <c r="F16" s="8"/>
+      <c r="G16" s="11">
         <v>0</v>
       </c>
-      <c r="I16">
+      <c r="H16" s="8"/>
+      <c r="I16" s="11">
         <v>0</v>
       </c>
-      <c r="J16" s="9">
+      <c r="J16" s="12">
         <v>1382549.88</v>
       </c>
     </row>
     <row r="17" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="B17" s="5">
+      <c r="A17" s="9">
         <v>46314</v>
       </c>
-      <c r="C17" s="9">
+      <c r="B17" s="10">
         <v>336565.44</v>
       </c>
-      <c r="D17">
+      <c r="C17" s="11">
         <v>0</v>
       </c>
-      <c r="F17">
+      <c r="D17" s="8"/>
+      <c r="E17" s="11">
         <v>0</v>
       </c>
-      <c r="H17">
+      <c r="F17" s="8"/>
+      <c r="G17" s="11">
         <v>0</v>
       </c>
-      <c r="I17">
+      <c r="H17" s="8"/>
+      <c r="I17" s="11">
         <v>0</v>
       </c>
-      <c r="J17" s="9">
+      <c r="J17" s="12">
         <v>336565.44</v>
       </c>
     </row>
     <row r="18" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="B18" s="5">
+      <c r="A18" s="9">
         <v>46315</v>
       </c>
-      <c r="C18" s="9">
+      <c r="B18" s="10">
         <v>381768.26</v>
       </c>
-      <c r="D18" s="9">
+      <c r="C18" s="10">
         <v>-63152.34</v>
       </c>
-      <c r="E18" s="9">
+      <c r="D18" s="10">
         <v>51209.3</v>
       </c>
-      <c r="F18">
+      <c r="E18" s="11">
         <v>0</v>
       </c>
-      <c r="H18">
+      <c r="F18" s="8"/>
+      <c r="G18" s="11">
         <v>0</v>
       </c>
-      <c r="I18">
+      <c r="H18" s="8"/>
+      <c r="I18" s="11">
         <v>0</v>
       </c>
-      <c r="J18" s="9">
+      <c r="J18" s="12">
         <v>369825.22</v>
       </c>
     </row>
     <row r="19" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="B19" s="5">
+      <c r="A19" s="9">
         <v>46316</v>
       </c>
-      <c r="C19" s="9">
+      <c r="B19" s="10">
         <v>548968.22</v>
       </c>
-      <c r="D19" s="9">
+      <c r="C19" s="10">
         <v>-24640.94</v>
       </c>
-      <c r="E19" s="9">
+      <c r="D19" s="10">
         <v>43879.51</v>
       </c>
-      <c r="F19">
+      <c r="E19" s="11">
         <v>0</v>
       </c>
-      <c r="H19">
+      <c r="F19" s="8"/>
+      <c r="G19" s="11">
         <v>0</v>
       </c>
-      <c r="I19">
+      <c r="H19" s="8"/>
+      <c r="I19" s="11">
         <v>0</v>
       </c>
-      <c r="J19" s="9">
+      <c r="J19" s="12">
         <v>568206.79</v>
       </c>
     </row>
     <row r="20" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="B20" s="5">
+      <c r="A20" s="9">
         <v>46317</v>
       </c>
-      <c r="C20" s="9">
+      <c r="B20" s="10">
         <v>647160.07999999996</v>
       </c>
-      <c r="D20" s="9">
+      <c r="C20" s="10">
         <v>-26687.200000000001</v>
       </c>
-      <c r="E20" s="9">
+      <c r="D20" s="10">
         <v>50411.43</v>
       </c>
-      <c r="F20">
+      <c r="E20" s="11">
         <v>0</v>
       </c>
-      <c r="H20">
+      <c r="F20" s="8"/>
+      <c r="G20" s="11">
         <v>0</v>
       </c>
-      <c r="I20">
+      <c r="H20" s="8"/>
+      <c r="I20" s="11">
         <v>0</v>
       </c>
-      <c r="J20" s="9">
+      <c r="J20" s="12">
         <v>670884.31000000006</v>
       </c>
     </row>
     <row r="21" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="B21" s="5">
+      <c r="A21" s="9">
         <v>46318</v>
       </c>
-      <c r="C21" s="9">
+      <c r="B21" s="10">
         <v>380210.58</v>
       </c>
-      <c r="D21" s="9">
+      <c r="C21" s="10">
         <v>-19833.009999999998</v>
       </c>
-      <c r="E21" s="9">
+      <c r="D21" s="10">
         <v>22362.76</v>
       </c>
-      <c r="F21">
+      <c r="E21" s="11">
         <v>0</v>
       </c>
-      <c r="H21">
+      <c r="F21" s="8"/>
+      <c r="G21" s="11">
         <v>0</v>
       </c>
-      <c r="I21">
+      <c r="H21" s="8"/>
+      <c r="I21" s="11">
         <v>0</v>
       </c>
-      <c r="J21" s="9">
+      <c r="J21" s="12">
         <v>382740.33</v>
       </c>
     </row>
     <row r="22" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="B22" s="5">
+      <c r="A22" s="9">
         <v>46321</v>
       </c>
-      <c r="C22" s="9">
+      <c r="B22" s="10">
         <v>833062.77</v>
       </c>
-      <c r="D22" s="9">
+      <c r="C22" s="10">
         <v>-8601.89</v>
       </c>
-      <c r="E22" s="9">
+      <c r="D22" s="10">
         <v>30850.26</v>
       </c>
-      <c r="F22">
+      <c r="E22" s="11">
         <v>0</v>
       </c>
-      <c r="H22">
+      <c r="F22" s="8"/>
+      <c r="G22" s="11">
         <v>0</v>
       </c>
-      <c r="I22">
+      <c r="H22" s="8"/>
+      <c r="I22" s="11">
         <v>0</v>
       </c>
-      <c r="J22" s="9">
+      <c r="J22" s="12">
         <v>855311.14</v>
       </c>
     </row>
     <row r="23" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="B23" s="5">
+      <c r="A23" s="9">
         <v>46322</v>
       </c>
-      <c r="C23" s="9">
+      <c r="B23" s="10">
         <v>403142.18</v>
       </c>
-      <c r="D23">
+      <c r="C23" s="11">
         <v>-397.64</v>
       </c>
-      <c r="E23" s="9">
+      <c r="D23" s="10">
         <v>15633.35</v>
       </c>
-      <c r="F23" s="9">
+      <c r="E23" s="10">
         <v>-4776.72</v>
       </c>
-      <c r="H23">
+      <c r="F23" s="8"/>
+      <c r="G23" s="11">
         <v>0</v>
       </c>
-      <c r="I23">
+      <c r="H23" s="8"/>
+      <c r="I23" s="11">
         <v>0</v>
       </c>
-      <c r="J23" s="9">
+      <c r="J23" s="12">
         <v>413601.17</v>
       </c>
     </row>
     <row r="24" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="B24" s="5">
+      <c r="A24" s="9">
         <v>46323</v>
       </c>
-      <c r="C24" s="9">
+      <c r="B24" s="10">
         <v>367755.97</v>
       </c>
-      <c r="D24" s="9">
+      <c r="C24" s="10">
         <v>-14081.69</v>
       </c>
-      <c r="E24" s="9">
+      <c r="D24" s="10">
         <v>20991.67</v>
       </c>
-      <c r="F24">
+      <c r="E24" s="11">
         <v>0</v>
       </c>
-      <c r="H24">
+      <c r="F24" s="8"/>
+      <c r="G24" s="11">
         <v>0</v>
       </c>
-      <c r="I24">
+      <c r="H24" s="8"/>
+      <c r="I24" s="11">
         <v>0</v>
       </c>
-      <c r="J24" s="9">
+      <c r="J24" s="12">
         <v>374665.95</v>
       </c>
     </row>
     <row r="25" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="B25" s="5">
+      <c r="A25" s="9">
         <v>46324</v>
       </c>
-      <c r="C25" s="9">
+      <c r="B25" s="10">
         <v>39248.85</v>
       </c>
-      <c r="D25" s="9">
+      <c r="C25" s="10">
         <v>-30205.25</v>
       </c>
-      <c r="F25">
+      <c r="D25" s="8"/>
+      <c r="E25" s="11">
         <v>0</v>
       </c>
-      <c r="H25">
+      <c r="F25" s="8"/>
+      <c r="G25" s="11">
         <v>0</v>
       </c>
-      <c r="I25">
+      <c r="H25" s="8"/>
+      <c r="I25" s="11">
         <v>0</v>
       </c>
-      <c r="J25" s="9">
+      <c r="J25" s="12">
+        <v>9043.6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="14">
+        <v>9509365.8000000007</v>
+      </c>
+      <c r="C26" s="14">
+        <v>-364063.73</v>
+      </c>
+      <c r="D26" s="14">
+        <v>660657.04</v>
+      </c>
+      <c r="E26" s="14">
+        <v>-16328.66</v>
+      </c>
+      <c r="F26" s="15">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" t="s">
-        <v>75</v>
-      </c>
-      <c r="C26" s="9">
-        <v>9509365.8000000007</v>
-      </c>
-      <c r="D26" s="9">
-        <v>-364063.73</v>
-      </c>
-      <c r="E26" s="9">
-        <v>660657.04</v>
-      </c>
-      <c r="F26" s="9">
-        <v>-16328.66</v>
-      </c>
-      <c r="G26">
+      <c r="G26" s="15">
         <v>0</v>
       </c>
-      <c r="H26">
+      <c r="H26" s="15">
         <v>0</v>
       </c>
-      <c r="I26">
+      <c r="I26" s="15">
         <v>0</v>
       </c>
-      <c r="J26" s="9">
+      <c r="J26" s="14">
         <v>9789630.4499999993</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
+    <mergeCell ref="J1:J2"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="F1:G1"/>
+    <mergeCell ref="A1:A2"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B3" r:id="rId1" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=01%2F10%2F2026&amp;wDT_FIM=01%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{687BB916-39E4-451A-9FD6-05CE7101E56A}"/>
+    <hyperlink ref="C3" r:id="rId2" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=01%2F10%2F2026&amp;wDT_FIM=01%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{E5FBD46F-E11A-4D2A-B9FE-F8CBC1E01A94}"/>
+    <hyperlink ref="D3" r:id="rId3" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=01%2F10%2F2026&amp;wDT_FIM=01%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{C706EFF1-19C6-43DB-BF1C-D774D72D3CE5}"/>
+    <hyperlink ref="E3" r:id="rId4" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=01%2F10%2F2026&amp;wDT_FIM=01%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{1315EF9F-1F25-4041-BC16-DE12039BA3CB}"/>
+    <hyperlink ref="G3" r:id="rId5" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=01%2F10%2F2026&amp;wDT_FIM=01%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{A9A8307D-310D-45BF-BF45-B21473727FC3}"/>
+    <hyperlink ref="I3" r:id="rId6" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=01%2F10%2F2026&amp;wDT_FIM=01%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{4C2DAC39-BD81-43B0-8EA7-456B2BB9799B}"/>
+    <hyperlink ref="B4" r:id="rId7" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=02%2F10%2F2026&amp;wDT_FIM=02%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{9DAF6DFA-76E5-4514-A106-958279A2DC2C}"/>
+    <hyperlink ref="C4" r:id="rId8" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=02%2F10%2F2026&amp;wDT_FIM=02%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{097FE572-AFA1-47B0-90CE-FE32B44A7B66}"/>
+    <hyperlink ref="D4" r:id="rId9" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=02%2F10%2F2026&amp;wDT_FIM=02%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{1E17B66C-D739-4BCE-A5F7-04A6F0EE91BD}"/>
+    <hyperlink ref="E4" r:id="rId10" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=02%2F10%2F2026&amp;wDT_FIM=02%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{78ECE9C6-7AC3-45E1-ADED-A8ED3C9BB380}"/>
+    <hyperlink ref="G4" r:id="rId11" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=02%2F10%2F2026&amp;wDT_FIM=02%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{B6C7B5F4-DB18-4CBF-902E-8D08E939B9C0}"/>
+    <hyperlink ref="I4" r:id="rId12" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=02%2F10%2F2026&amp;wDT_FIM=02%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{070523A6-7BBA-45A0-91A1-DD10E096AC83}"/>
+    <hyperlink ref="B5" r:id="rId13" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=05%2F10%2F2026&amp;wDT_FIM=05%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{A6FE5CE1-9AFF-43A0-A2F7-A5FA64AE1C82}"/>
+    <hyperlink ref="C5" r:id="rId14" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=05%2F10%2F2026&amp;wDT_FIM=05%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{5F06682F-785F-48AF-A556-9CB62F556813}"/>
+    <hyperlink ref="D5" r:id="rId15" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=05%2F10%2F2026&amp;wDT_FIM=05%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{99AECBC6-376B-463D-ABB3-613E6F334936}"/>
+    <hyperlink ref="E5" r:id="rId16" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=05%2F10%2F2026&amp;wDT_FIM=05%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{27865420-50C6-4B05-A8F7-78B1FC151DB8}"/>
+    <hyperlink ref="G5" r:id="rId17" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=05%2F10%2F2026&amp;wDT_FIM=05%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{3C074977-FBF5-40B5-995F-3B3FBDF4D757}"/>
+    <hyperlink ref="I5" r:id="rId18" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=05%2F10%2F2026&amp;wDT_FIM=05%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{942165DF-39D9-4890-BC49-3DC9CF408E78}"/>
+    <hyperlink ref="B6" r:id="rId19" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=06%2F10%2F2026&amp;wDT_FIM=06%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{BCC79D74-CE54-4820-A276-F1F847F0E585}"/>
+    <hyperlink ref="C6" r:id="rId20" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=06%2F10%2F2026&amp;wDT_FIM=06%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F7217115-1ED7-4776-838B-2EBAC408CA87}"/>
+    <hyperlink ref="D6" r:id="rId21" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=06%2F10%2F2026&amp;wDT_FIM=06%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{0C834F42-8441-4D44-A5F6-2E057DAA850C}"/>
+    <hyperlink ref="E6" r:id="rId22" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=06%2F10%2F2026&amp;wDT_FIM=06%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{82310EFD-5CCC-411D-AAD6-3D10203E31AE}"/>
+    <hyperlink ref="G6" r:id="rId23" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=06%2F10%2F2026&amp;wDT_FIM=06%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{0FBB09BD-6B32-40FA-9B50-16465E596A73}"/>
+    <hyperlink ref="I6" r:id="rId24" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=06%2F10%2F2026&amp;wDT_FIM=06%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{C015B2D3-473D-4B27-AA32-C1EB96A98E2F}"/>
+    <hyperlink ref="B7" r:id="rId25" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=07%2F10%2F2026&amp;wDT_FIM=07%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{D8B51840-FE95-4575-9F58-A14A89D1CC89}"/>
+    <hyperlink ref="C7" r:id="rId26" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=07%2F10%2F2026&amp;wDT_FIM=07%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{913B7A06-A561-49D9-9054-6988583CE0CF}"/>
+    <hyperlink ref="D7" r:id="rId27" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=07%2F10%2F2026&amp;wDT_FIM=07%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{5928DE69-8B49-4938-8BC0-2591C24A59DA}"/>
+    <hyperlink ref="E7" r:id="rId28" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=07%2F10%2F2026&amp;wDT_FIM=07%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{6A64E255-EAEC-4015-92E3-718673D24F41}"/>
+    <hyperlink ref="G7" r:id="rId29" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=07%2F10%2F2026&amp;wDT_FIM=07%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{171A8010-629F-4FCF-A267-F8977772A919}"/>
+    <hyperlink ref="I7" r:id="rId30" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=07%2F10%2F2026&amp;wDT_FIM=07%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{84D00DCA-8910-488F-A8BE-CF00F1AA773D}"/>
+    <hyperlink ref="B8" r:id="rId31" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=08%2F10%2F2026&amp;wDT_FIM=08%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{8A4AF581-4EA9-4887-9BA9-7B71127B5BEE}"/>
+    <hyperlink ref="C8" r:id="rId32" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=08%2F10%2F2026&amp;wDT_FIM=08%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{FA63E263-C6EB-47FB-BB42-744574F43B36}"/>
+    <hyperlink ref="D8" r:id="rId33" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=08%2F10%2F2026&amp;wDT_FIM=08%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{46A855A0-B703-4A32-855A-133544FFA78E}"/>
+    <hyperlink ref="E8" r:id="rId34" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=08%2F10%2F2026&amp;wDT_FIM=08%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{81269BBD-6466-47BA-8954-B99AB7E547FD}"/>
+    <hyperlink ref="G8" r:id="rId35" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=08%2F10%2F2026&amp;wDT_FIM=08%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{8D159887-6B6B-4CF0-B136-959762FC53E5}"/>
+    <hyperlink ref="I8" r:id="rId36" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=08%2F10%2F2026&amp;wDT_FIM=08%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{AC9BAAD9-DB01-4874-A326-3ECFFE2AB771}"/>
+    <hyperlink ref="B9" r:id="rId37" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=09%2F10%2F2026&amp;wDT_FIM=09%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{ADECEC3D-1503-432D-9CE7-1D303F2EDA65}"/>
+    <hyperlink ref="C9" r:id="rId38" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=09%2F10%2F2026&amp;wDT_FIM=09%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{3DDFFF8C-7C65-4049-8FB5-880E5FAD2015}"/>
+    <hyperlink ref="D9" r:id="rId39" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=09%2F10%2F2026&amp;wDT_FIM=09%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{B6B2BAD8-9818-4A17-B2AF-5EB790564079}"/>
+    <hyperlink ref="E9" r:id="rId40" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=09%2F10%2F2026&amp;wDT_FIM=09%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{C3B9EC01-61F5-4418-9557-82EDCF8B1547}"/>
+    <hyperlink ref="G9" r:id="rId41" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=09%2F10%2F2026&amp;wDT_FIM=09%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{910F2F42-170A-4154-95A4-D576BF7E7119}"/>
+    <hyperlink ref="I9" r:id="rId42" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=09%2F10%2F2026&amp;wDT_FIM=09%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{73B71715-8B25-4802-A48B-206FEAB99577}"/>
+    <hyperlink ref="B10" r:id="rId43" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=10%2F10%2F2026&amp;wDT_FIM=10%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{1FFD6E12-D3BE-4FA7-A788-72E75A84EE48}"/>
+    <hyperlink ref="C10" r:id="rId44" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=10%2F10%2F2026&amp;wDT_FIM=10%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{60F13880-8519-4548-9073-F64C0E729464}"/>
+    <hyperlink ref="E10" r:id="rId45" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=10%2F10%2F2026&amp;wDT_FIM=10%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F2031124-7203-4B15-9E34-960BD3FC4AB9}"/>
+    <hyperlink ref="G10" r:id="rId46" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=10%2F10%2F2026&amp;wDT_FIM=10%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{39CCCDF7-0082-4581-9A5C-D7A3626EF94A}"/>
+    <hyperlink ref="I10" r:id="rId47" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=10%2F10%2F2026&amp;wDT_FIM=10%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{0389E5D8-2ECA-4149-A985-3C38E758D9A5}"/>
+    <hyperlink ref="B11" r:id="rId48" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=11%2F10%2F2026&amp;wDT_FIM=11%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{30B1B3A3-0004-4192-B744-3D6C29732962}"/>
+    <hyperlink ref="C11" r:id="rId49" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=11%2F10%2F2026&amp;wDT_FIM=11%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{8DD9D58B-DC7C-4DDE-B29B-1A191FCC27EC}"/>
+    <hyperlink ref="E11" r:id="rId50" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=11%2F10%2F2026&amp;wDT_FIM=11%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{6DD58EF5-84D0-43E6-8308-38241B6F33A6}"/>
+    <hyperlink ref="G11" r:id="rId51" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=11%2F10%2F2026&amp;wDT_FIM=11%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{8FDEFA51-3826-4AC9-B413-AB809828CC27}"/>
+    <hyperlink ref="I11" r:id="rId52" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=11%2F10%2F2026&amp;wDT_FIM=11%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{29EAB79F-E12E-4CA1-B0A4-5371C4363F2E}"/>
+    <hyperlink ref="B12" r:id="rId53" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=12%2F10%2F2026&amp;wDT_FIM=12%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{CED61254-7A53-4676-8894-8527F0937B26}"/>
+    <hyperlink ref="C12" r:id="rId54" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=12%2F10%2F2026&amp;wDT_FIM=12%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{FB0C6349-F7A9-44BE-8D7C-BC51053FCFA0}"/>
+    <hyperlink ref="E12" r:id="rId55" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=12%2F10%2F2026&amp;wDT_FIM=12%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{001031EB-4A3F-486C-B2E9-E90310B771B2}"/>
+    <hyperlink ref="G12" r:id="rId56" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=12%2F10%2F2026&amp;wDT_FIM=12%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{329980CD-A0C3-49B7-8A0F-151CBF8D346F}"/>
+    <hyperlink ref="I12" r:id="rId57" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=12%2F10%2F2026&amp;wDT_FIM=12%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{BA8C7164-B9AC-453C-AC13-390EF76C3CAA}"/>
+    <hyperlink ref="B13" r:id="rId58" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=13%2F10%2F2026&amp;wDT_FIM=13%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{04B51785-D512-4943-AE8C-0D8BE107D63D}"/>
+    <hyperlink ref="C13" r:id="rId59" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=13%2F10%2F2026&amp;wDT_FIM=13%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{FD9277CC-07A3-444D-AA93-AE4686F3DDD2}"/>
+    <hyperlink ref="D13" r:id="rId60" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=13%2F10%2F2026&amp;wDT_FIM=13%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{82C93853-7B6E-4349-BEF6-D6743752A55B}"/>
+    <hyperlink ref="E13" r:id="rId61" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=13%2F10%2F2026&amp;wDT_FIM=13%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{BE630531-0E43-4541-9855-02D96EA186CF}"/>
+    <hyperlink ref="G13" r:id="rId62" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=13%2F10%2F2026&amp;wDT_FIM=13%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{780AD855-20EC-46E0-8309-4927B05D52C0}"/>
+    <hyperlink ref="I13" r:id="rId63" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=13%2F10%2F2026&amp;wDT_FIM=13%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{0F397AE1-7108-4873-98AA-42DF29077EBA}"/>
+    <hyperlink ref="B14" r:id="rId64" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=14%2F10%2F2026&amp;wDT_FIM=14%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{69984AF0-BFBD-4576-AAB7-E720EB47AA23}"/>
+    <hyperlink ref="C14" r:id="rId65" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=14%2F10%2F2026&amp;wDT_FIM=14%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{E741674C-9639-4284-85DA-2758B4B98186}"/>
+    <hyperlink ref="D14" r:id="rId66" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=14%2F10%2F2026&amp;wDT_FIM=14%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{0EAB373F-90CB-4781-881A-18B44C5C67CE}"/>
+    <hyperlink ref="E14" r:id="rId67" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=14%2F10%2F2026&amp;wDT_FIM=14%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{C9950F5F-F47E-4017-BD4C-CB6C5E1AD4EA}"/>
+    <hyperlink ref="G14" r:id="rId68" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=14%2F10%2F2026&amp;wDT_FIM=14%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{9ED67B91-146B-4BA0-89AF-12E3B525B057}"/>
+    <hyperlink ref="I14" r:id="rId69" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=14%2F10%2F2026&amp;wDT_FIM=14%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{75091688-CCD1-4148-8302-C16C62A3ECEB}"/>
+    <hyperlink ref="B15" r:id="rId70" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=15%2F10%2F2026&amp;wDT_FIM=15%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{51AB3956-06F7-42FF-92F7-87725F4628B9}"/>
+    <hyperlink ref="C15" r:id="rId71" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=15%2F10%2F2026&amp;wDT_FIM=15%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{D01B4EA1-DE0E-4C8E-9A83-0611A7BC37EE}"/>
+    <hyperlink ref="D15" r:id="rId72" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=15%2F10%2F2026&amp;wDT_FIM=15%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{A9DE5639-D4AC-4A1B-B83A-DEFF954978CA}"/>
+    <hyperlink ref="E15" r:id="rId73" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=15%2F10%2F2026&amp;wDT_FIM=15%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{5BBB9CFD-24F5-4F9B-8C3B-D385341FB79F}"/>
+    <hyperlink ref="G15" r:id="rId74" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=15%2F10%2F2026&amp;wDT_FIM=15%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{E633D1D4-CA93-4115-B984-F66B88BF3416}"/>
+    <hyperlink ref="I15" r:id="rId75" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=15%2F10%2F2026&amp;wDT_FIM=15%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{13357E6C-BB30-484B-8400-F91EE2A7D07E}"/>
+    <hyperlink ref="B16" r:id="rId76" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=16%2F10%2F2026&amp;wDT_FIM=16%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{057E90F7-6A40-4EDE-9A3E-F30A859CF3BE}"/>
+    <hyperlink ref="C16" r:id="rId77" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=16%2F10%2F2026&amp;wDT_FIM=16%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F7DB2805-0CDB-484E-B723-B80837A45A7C}"/>
+    <hyperlink ref="D16" r:id="rId78" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=16%2F10%2F2026&amp;wDT_FIM=16%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{47E74C81-3114-45F2-986C-956A43348F2B}"/>
+    <hyperlink ref="E16" r:id="rId79" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=16%2F10%2F2026&amp;wDT_FIM=16%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{55782F92-7117-4BA1-BB3C-7206EDDCE433}"/>
+    <hyperlink ref="G16" r:id="rId80" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=16%2F10%2F2026&amp;wDT_FIM=16%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{A2A6CF9B-8818-4C36-9182-BB4C1CD6E24D}"/>
+    <hyperlink ref="I16" r:id="rId81" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=16%2F10%2F2026&amp;wDT_FIM=16%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{4A7E4F9B-D384-4C96-9E21-EF9427F927A0}"/>
+    <hyperlink ref="B17" r:id="rId82" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=19%2F10%2F2026&amp;wDT_FIM=19%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{93C9F410-EA82-4975-A9CA-E8E7C9E6E495}"/>
+    <hyperlink ref="C17" r:id="rId83" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=19%2F10%2F2026&amp;wDT_FIM=19%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{A261D0F3-D257-498A-916F-FC902A0B02BA}"/>
+    <hyperlink ref="E17" r:id="rId84" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=19%2F10%2F2026&amp;wDT_FIM=19%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{6F6EF0DF-0CDA-4824-B98D-C894AFE2F645}"/>
+    <hyperlink ref="G17" r:id="rId85" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=19%2F10%2F2026&amp;wDT_FIM=19%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{A64E6B0D-5609-420E-A0F9-2CD8282DF21E}"/>
+    <hyperlink ref="I17" r:id="rId86" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=19%2F10%2F2026&amp;wDT_FIM=19%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F1155477-B7F0-421A-9F9F-26636A548949}"/>
+    <hyperlink ref="B18" r:id="rId87" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=20%2F10%2F2026&amp;wDT_FIM=20%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{63B925F4-B927-4D4B-AF30-932AEBEE9398}"/>
+    <hyperlink ref="C18" r:id="rId88" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=20%2F10%2F2026&amp;wDT_FIM=20%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{13B50C12-A016-4095-80AB-9C31F37F9631}"/>
+    <hyperlink ref="D18" r:id="rId89" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=20%2F10%2F2026&amp;wDT_FIM=20%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{6CE45C78-33FF-409B-B7D1-55ED5243215C}"/>
+    <hyperlink ref="E18" r:id="rId90" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=20%2F10%2F2026&amp;wDT_FIM=20%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F81D7FAA-6209-4009-8307-F99F7A8A264B}"/>
+    <hyperlink ref="G18" r:id="rId91" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=20%2F10%2F2026&amp;wDT_FIM=20%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{5E4EE0FA-B3A6-4483-8853-49B026528B1C}"/>
+    <hyperlink ref="I18" r:id="rId92" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=20%2F10%2F2026&amp;wDT_FIM=20%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{5805841B-46C8-4811-A12A-93F1DF772040}"/>
+    <hyperlink ref="B19" r:id="rId93" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=21%2F10%2F2026&amp;wDT_FIM=21%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{879CA852-48F7-47EA-8032-E11E92617195}"/>
+    <hyperlink ref="C19" r:id="rId94" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=21%2F10%2F2026&amp;wDT_FIM=21%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{C341E091-4BE7-44D7-94C5-24322C9FB854}"/>
+    <hyperlink ref="D19" r:id="rId95" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=21%2F10%2F2026&amp;wDT_FIM=21%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{BD6A736D-E57D-4E62-8311-AD3B2D3789E1}"/>
+    <hyperlink ref="E19" r:id="rId96" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=21%2F10%2F2026&amp;wDT_FIM=21%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{E8FA1758-0AB6-4D9C-970A-0EF3A77B867A}"/>
+    <hyperlink ref="G19" r:id="rId97" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=21%2F10%2F2026&amp;wDT_FIM=21%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F817A03E-2763-4E40-A607-DB36EDA79830}"/>
+    <hyperlink ref="I19" r:id="rId98" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=21%2F10%2F2026&amp;wDT_FIM=21%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{25CAEB8F-B63C-484E-BC45-F81165558C94}"/>
+    <hyperlink ref="B20" r:id="rId99" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=22%2F10%2F2026&amp;wDT_FIM=22%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{7DA6DE3B-61E7-4299-8BC4-FC2AF3E662F8}"/>
+    <hyperlink ref="C20" r:id="rId100" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=22%2F10%2F2026&amp;wDT_FIM=22%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{BD60FEF0-5474-46D6-A5F2-EF2DAFF8B99B}"/>
+    <hyperlink ref="D20" r:id="rId101" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=22%2F10%2F2026&amp;wDT_FIM=22%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{49D3EB46-3608-49B9-A55C-96E319E31E51}"/>
+    <hyperlink ref="E20" r:id="rId102" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=22%2F10%2F2026&amp;wDT_FIM=22%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F088F589-3D39-42DA-AF41-25DDB3728F24}"/>
+    <hyperlink ref="G20" r:id="rId103" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=22%2F10%2F2026&amp;wDT_FIM=22%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F3C47B57-3594-4D55-A617-FFDC13F5FB73}"/>
+    <hyperlink ref="I20" r:id="rId104" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=22%2F10%2F2026&amp;wDT_FIM=22%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{1FC47A20-9CE2-4784-B0BA-E38A9864DCE4}"/>
+    <hyperlink ref="B21" r:id="rId105" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{E319463A-8363-4BBA-B1A3-39F493B7B6D9}"/>
+    <hyperlink ref="C21" r:id="rId106" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{57A685E2-9D7A-4021-822F-26463A7EEA54}"/>
+    <hyperlink ref="D21" r:id="rId107" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{4976344E-0814-4EFE-AB2F-EE2FE3AF2C2E}"/>
+    <hyperlink ref="E21" r:id="rId108" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{695CE89C-574C-4A69-B7B7-7FF03B4CD7B1}"/>
+    <hyperlink ref="G21" r:id="rId109" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F86D88F9-D317-461D-9C61-FF135999D175}"/>
+    <hyperlink ref="I21" r:id="rId110" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=23%2F10%2F2026&amp;wDT_FIM=23%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{D0326386-67B6-4488-A438-F8FBAC6A450F}"/>
+    <hyperlink ref="B22" r:id="rId111" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{C7AF566F-9632-4AA4-8F34-0B970597D3BA}"/>
+    <hyperlink ref="C22" r:id="rId112" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{169EAA2C-A6AC-4FCE-93BB-ACEF1B3F8EBC}"/>
+    <hyperlink ref="D22" r:id="rId113" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{7676174D-27EF-49A8-A14E-D7BC7E0216B1}"/>
+    <hyperlink ref="E22" r:id="rId114" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{24DB1586-F850-47B7-9679-1296B90D21FF}"/>
+    <hyperlink ref="G22" r:id="rId115" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F6EE7820-E235-40AE-9EE0-D9FF248828DF}"/>
+    <hyperlink ref="I22" r:id="rId116" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=26%2F10%2F2026&amp;wDT_FIM=26%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{59D0B290-8208-4530-9196-E059E3EFB104}"/>
+    <hyperlink ref="B23" r:id="rId117" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{8A006336-1515-4366-BB60-0F379AB25E3D}"/>
+    <hyperlink ref="C23" r:id="rId118" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{B27C3982-31D4-4CAD-A4BF-03134A481775}"/>
+    <hyperlink ref="D23" r:id="rId119" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{7A7748FF-DCEF-4FE1-9493-4A90724AD4B8}"/>
+    <hyperlink ref="E23" r:id="rId120" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{93532439-7A0E-4DEA-B3D9-0784C51E7BE7}"/>
+    <hyperlink ref="G23" r:id="rId121" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{0DC2FEC9-B20A-401A-8D11-AC1D2F0DC61B}"/>
+    <hyperlink ref="I23" r:id="rId122" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=27%2F10%2F2026&amp;wDT_FIM=27%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{0FD5E040-B03A-455A-9204-5AAD0A2AED19}"/>
+    <hyperlink ref="B24" r:id="rId123" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{D44FD28B-EBF8-471F-BB31-1BEFD1F43233}"/>
+    <hyperlink ref="C24" r:id="rId124" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{9EAB19A3-BECE-4184-930C-6A15ED9A29D6}"/>
+    <hyperlink ref="D24" r:id="rId125" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{9D649A28-9791-4AAC-B0A1-F2C3CA303F0C}"/>
+    <hyperlink ref="E24" r:id="rId126" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{21823261-B4F4-47FA-86BC-5F7CEE4685B2}"/>
+    <hyperlink ref="G24" r:id="rId127" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{FB38D098-8B1C-43C1-AD3A-C194FB3E3C7F}"/>
+    <hyperlink ref="I24" r:id="rId128" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{14A793E0-75A1-4F59-9C35-B1536EC89BEF}"/>
+    <hyperlink ref="B25" r:id="rId129" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{26C339CF-03A2-4044-B71F-1B100CC059A9}"/>
+    <hyperlink ref="C25" r:id="rId130" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{02C307C1-145D-41B7-B1AE-A8080C58C1BE}"/>
+    <hyperlink ref="E25" r:id="rId131" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{18C8549A-2C10-4784-8559-867EC840A426}"/>
+    <hyperlink ref="G25" r:id="rId132" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{42E3BB6E-E58A-4D99-B8A0-A7FED1A97F48}"/>
+    <hyperlink ref="I25" r:id="rId133" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{93DD70DD-B00E-43A1-98BC-B520BE0CEE83}"/>
+  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId134"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: Correção de algumas falhas e campos
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47D6FC34-69BE-420C-B4F6-814AC15640A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{984F8F84-D9C0-49F4-B5AE-75BA115EA04B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
@@ -16,12 +16,25 @@
     <sheet name="FaturamentoBruto" sheetId="1" r:id="rId1"/>
     <sheet name="Faturamento por cliente" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="253">
   <si>
     <t>Filial</t>
   </si>
@@ -777,6 +790,9 @@
   </si>
   <si>
     <t>TOT</t>
+  </si>
+  <si>
+    <t>DEV</t>
   </si>
 </sst>
 </file>
@@ -1467,10 +1483,10 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1479,10 +1495,10 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1860,7 +1876,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19101EBF-008C-4E37-90C0-CF2D419D5300}">
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr defaultRowHeight="15.75" thickBottom="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -1871,10 +1887,11 @@
     <col min="7" max="7" width="11.140625" customWidth="1"/>
     <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="20" t="s">
         <v>76</v>
       </c>
       <c r="B1" s="18" t="s">
@@ -1893,12 +1910,15 @@
         <v>250</v>
       </c>
       <c r="I1" s="19"/>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="16" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="17"/>
+      <c r="K1" s="16" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="21"/>
       <c r="B2" s="7" t="s">
         <v>78</v>
       </c>
@@ -1923,9 +1943,10 @@
       <c r="I2" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="J2" s="21"/>
-    </row>
-    <row r="3" spans="1:10" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+    </row>
+    <row r="3" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9">
         <v>46296</v>
       </c>
@@ -1952,8 +1973,12 @@
       <c r="J3" s="12">
         <v>272046.58</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K3" s="12">
+        <f>SUM(C3+E3+G3+I3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9">
         <v>46297</v>
       </c>
@@ -1980,8 +2005,12 @@
       <c r="J4" s="12">
         <v>457346.52</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K4" s="12">
+        <f t="shared" ref="K4:K26" si="0">SUM(C4+E4+G4+I4)</f>
+        <v>-26599.88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9">
         <v>46300</v>
       </c>
@@ -2008,8 +2037,12 @@
       <c r="J5" s="12">
         <v>305376.46000000002</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K5" s="12">
+        <f t="shared" si="0"/>
+        <v>-7502.05</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9">
         <v>46301</v>
       </c>
@@ -2036,8 +2069,12 @@
       <c r="J6" s="12">
         <v>461218.26</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K6" s="12">
+        <f t="shared" si="0"/>
+        <v>-15592.96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9">
         <v>46302</v>
       </c>
@@ -2064,8 +2101,12 @@
       <c r="J7" s="12">
         <v>319812.01</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K7" s="12">
+        <f t="shared" si="0"/>
+        <v>-12949.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9">
         <v>46303</v>
       </c>
@@ -2092,8 +2133,12 @@
       <c r="J8" s="12">
         <v>592806.96</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K8" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
         <v>46304</v>
       </c>
@@ -2120,8 +2165,12 @@
       <c r="J9" s="12">
         <v>283538.15000000002</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K9" s="12">
+        <f t="shared" si="0"/>
+        <v>-70683.45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9">
         <v>46305</v>
       </c>
@@ -2146,8 +2195,12 @@
       <c r="J10" s="12">
         <v>203772.98</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K10" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="9">
         <v>46306</v>
       </c>
@@ -2172,8 +2225,12 @@
       <c r="J11" s="12">
         <v>169560.7</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K11" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9">
         <v>46307</v>
       </c>
@@ -2198,8 +2255,12 @@
       <c r="J12" s="12">
         <v>216275.07</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K12" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="9">
         <v>46308</v>
       </c>
@@ -2226,8 +2287,12 @@
       <c r="J13" s="12">
         <v>504715.42</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K13" s="12">
+        <f t="shared" si="0"/>
+        <v>-29468.28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="9">
         <v>46309</v>
       </c>
@@ -2254,8 +2319,12 @@
       <c r="J14" s="12">
         <v>335630.1</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K14" s="12">
+        <f t="shared" si="0"/>
+        <v>-14134.51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="9">
         <v>46310</v>
       </c>
@@ -2282,8 +2351,12 @@
       <c r="J15" s="12">
         <v>304137.40999999997</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K15" s="12">
+        <f t="shared" si="0"/>
+        <v>-11085.38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="9">
         <v>46311</v>
       </c>
@@ -2310,8 +2383,12 @@
       <c r="J16" s="12">
         <v>1382549.88</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K16" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="9">
         <v>46314</v>
       </c>
@@ -2336,8 +2413,12 @@
       <c r="J17" s="12">
         <v>336565.44</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K17" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9">
         <v>46315</v>
       </c>
@@ -2364,8 +2445,12 @@
       <c r="J18" s="12">
         <v>369825.22</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K18" s="12">
+        <f t="shared" si="0"/>
+        <v>-63152.34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9">
         <v>46316</v>
       </c>
@@ -2392,8 +2477,12 @@
       <c r="J19" s="12">
         <v>568206.79</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K19" s="12">
+        <f t="shared" si="0"/>
+        <v>-24640.94</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="9">
         <v>46317</v>
       </c>
@@ -2420,8 +2509,12 @@
       <c r="J20" s="12">
         <v>670884.31000000006</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K20" s="12">
+        <f t="shared" si="0"/>
+        <v>-26687.200000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="9">
         <v>46318</v>
       </c>
@@ -2448,8 +2541,12 @@
       <c r="J21" s="12">
         <v>382740.33</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K21" s="12">
+        <f t="shared" si="0"/>
+        <v>-19833.009999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="9">
         <v>46321</v>
       </c>
@@ -2476,8 +2573,12 @@
       <c r="J22" s="12">
         <v>855311.14</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K22" s="12">
+        <f t="shared" si="0"/>
+        <v>-8601.89</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9">
         <v>46322</v>
       </c>
@@ -2504,8 +2605,12 @@
       <c r="J23" s="12">
         <v>413601.17</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K23" s="12">
+        <f t="shared" si="0"/>
+        <v>-5174.3600000000006</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="9">
         <v>46323</v>
       </c>
@@ -2532,8 +2637,12 @@
       <c r="J24" s="12">
         <v>374665.95</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K24" s="12">
+        <f t="shared" si="0"/>
+        <v>-14081.69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="9">
         <v>46324</v>
       </c>
@@ -2558,8 +2667,12 @@
       <c r="J25" s="12">
         <v>9043.6</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K25" s="12">
+        <f t="shared" si="0"/>
+        <v>-30205.25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="13" t="s">
         <v>75</v>
       </c>
@@ -2590,15 +2703,20 @@
       <c r="J26" s="14">
         <v>9789630.4499999993</v>
       </c>
+      <c r="K26" s="14">
+        <f>SUM(K3:K25)</f>
+        <v>-380392.39</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="K1:K2"/>
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="F1:G1"/>
-    <mergeCell ref="A1:A2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=01%2F10%2F2026&amp;wDT_FIM=01%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{687BB916-39E4-451A-9FD6-05CE7101E56A}"/>

</xml_diff>

<commit_message>
Segunda atualização dos dados e correção dos bugs
</commit_message>
<xml_diff>
--- a/DadosFaturamento.xlsx
+++ b/DadosFaturamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{984F8F84-D9C0-49F4-B5AE-75BA115EA04B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C9A479B-2D61-46ED-8C2B-F459B239B014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{CBC36103-499F-47D2-920C-CE20E86CCBE2}"/>
   </bookViews>
@@ -1164,7 +1164,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -1391,6 +1391,51 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDEE2E6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDEE2E6"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDEE2E6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDEE2E6"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1437,7 +1482,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="19" fillId="33" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1473,14 +1518,14 @@
     <xf numFmtId="4" fontId="22" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="4" fontId="21" fillId="34" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -1494,11 +1539,29 @@
     <xf numFmtId="0" fontId="21" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="19" fillId="33" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="20" fillId="33" borderId="19" xfId="42" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="19" xfId="42" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="19" fillId="33" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="4" fontId="18" fillId="34" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1886,12 +1949,12 @@
     <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.140625" customWidth="1"/>
     <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="14" t="s">
         <v>76</v>
       </c>
       <c r="B1" s="18" t="s">
@@ -1918,7 +1981,7 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="21"/>
+      <c r="A2" s="15"/>
       <c r="B2" s="7" t="s">
         <v>78</v>
       </c>
@@ -2006,7 +2069,7 @@
         <v>457346.52</v>
       </c>
       <c r="K4" s="12">
-        <f t="shared" ref="K4:K26" si="0">SUM(C4+E4+G4+I4)</f>
+        <f t="shared" ref="K4:K25" si="0">SUM(C4+E4+G4+I4)</f>
         <v>-26599.88</v>
       </c>
     </row>
@@ -2643,69 +2706,71 @@
       </c>
     </row>
     <row r="25" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="9">
+      <c r="A25" s="20">
         <v>46324</v>
       </c>
-      <c r="B25" s="10">
-        <v>39248.85</v>
-      </c>
-      <c r="C25" s="10">
-        <v>-30205.25</v>
-      </c>
-      <c r="D25" s="8"/>
-      <c r="E25" s="11">
+      <c r="B25" s="21">
+        <v>50832.02</v>
+      </c>
+      <c r="C25" s="21">
+        <v>-32762.45</v>
+      </c>
+      <c r="D25" s="21">
+        <v>11640.48</v>
+      </c>
+      <c r="E25" s="22">
         <v>0</v>
       </c>
-      <c r="F25" s="8"/>
-      <c r="G25" s="11">
+      <c r="F25" s="23"/>
+      <c r="G25" s="22">
         <v>0</v>
       </c>
-      <c r="H25" s="8"/>
-      <c r="I25" s="11">
+      <c r="H25" s="23"/>
+      <c r="I25" s="22">
         <v>0</v>
       </c>
-      <c r="J25" s="12">
-        <v>9043.6</v>
+      <c r="J25" s="24">
+        <v>29710.05</v>
       </c>
       <c r="K25" s="12">
         <f t="shared" si="0"/>
-        <v>-30205.25</v>
+        <v>-32762.45</v>
       </c>
     </row>
     <row r="26" spans="1:11" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="13" t="s">
+      <c r="A26" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="B26" s="14">
-        <v>9509365.8000000007</v>
-      </c>
-      <c r="C26" s="14">
-        <v>-364063.73</v>
-      </c>
-      <c r="D26" s="14">
-        <v>660657.04</v>
-      </c>
-      <c r="E26" s="14">
+      <c r="B26" s="26">
+        <v>9520948.9700000007</v>
+      </c>
+      <c r="C26" s="26">
+        <v>-366620.93</v>
+      </c>
+      <c r="D26" s="26">
+        <v>672297.52</v>
+      </c>
+      <c r="E26" s="26">
         <v>-16328.66</v>
       </c>
-      <c r="F26" s="15">
+      <c r="F26" s="27">
         <v>0</v>
       </c>
-      <c r="G26" s="15">
+      <c r="G26" s="27">
         <v>0</v>
       </c>
-      <c r="H26" s="15">
+      <c r="H26" s="27">
         <v>0</v>
       </c>
-      <c r="I26" s="15">
+      <c r="I26" s="27">
         <v>0</v>
       </c>
-      <c r="J26" s="14">
-        <v>9789630.4499999993</v>
-      </c>
-      <c r="K26" s="14">
+      <c r="J26" s="26">
+        <v>9810296.9000000004</v>
+      </c>
+      <c r="K26" s="13">
         <f>SUM(K3:K25)</f>
-        <v>-380392.39</v>
+        <v>-382949.59</v>
       </c>
     </row>
   </sheetData>
@@ -2847,14 +2912,15 @@
     <hyperlink ref="E24" r:id="rId126" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{21823261-B4F4-47FA-86BC-5F7CEE4685B2}"/>
     <hyperlink ref="G24" r:id="rId127" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{FB38D098-8B1C-43C1-AD3A-C194FB3E3C7F}"/>
     <hyperlink ref="I24" r:id="rId128" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=28%2F10%2F2026&amp;wDT_FIM=28%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{14A793E0-75A1-4F59-9C35-B1536EC89BEF}"/>
-    <hyperlink ref="B25" r:id="rId129" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{26C339CF-03A2-4044-B71F-1B100CC059A9}"/>
-    <hyperlink ref="C25" r:id="rId130" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{02C307C1-145D-41B7-B1AE-A8080C58C1BE}"/>
-    <hyperlink ref="E25" r:id="rId131" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{18C8549A-2C10-4784-8559-867EC840A426}"/>
-    <hyperlink ref="G25" r:id="rId132" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{42E3BB6E-E58A-4D99-B8A0-A7FED1A97F48}"/>
-    <hyperlink ref="I25" r:id="rId133" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{93DD70DD-B00E-43A1-98BC-B520BE0CEE83}"/>
+    <hyperlink ref="B25" r:id="rId129" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{6F9D287F-5B13-4F5E-B9A9-FAE3F21A9F05}"/>
+    <hyperlink ref="C25" r:id="rId130" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{E20DED4D-CA1D-4234-932E-9D0B5BFD88AA}"/>
+    <hyperlink ref="D25" r:id="rId131" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0102&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{93988AEF-44D8-440D-A3F9-80D13FDE9B8D}"/>
+    <hyperlink ref="E25" r:id="rId132" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{F30E50C5-74FA-474A-B0A5-1A1DA6C88237}"/>
+    <hyperlink ref="G25" r:id="rId133" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{B642C56F-47C6-4274-AB89-8D8203E0CC13}"/>
+    <hyperlink ref="I25" r:id="rId134" tooltip="por Cliente" display="https://qubex-higimed.integraerp.com.br/ViewCockpit001/Cp01Cli?wFIL_DD=0101&amp;wDT_INI=29%2F10%2F2026&amp;wDT_FIM=29%2F10%2F2026&amp;wACY_DD=%5B%22%2A%2A%2A%2A%2A%2A%22%5D" xr:uid="{C2C51E8D-EDDC-46DF-8B51-DB8FE9F897B0}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId134"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId135"/>
 </worksheet>
 </file>
 

</xml_diff>